<commit_message>
data: popola foglio Aziende del template Excel con 13 aziende dalla piattaforma
Aggiunge i dati reali di tutte le aziende attualmente presenti nel database
della piattaforma (companies-DS8bqSy6.js) nel foglio "Aziende" del file
MetaBorghi_DataTemplate.xlsx, come base di partenza per la raccolta dati reali.

Include anche lo script populate_excel.py usato per la migrazione.

https://claude.ai/code/session_018oe8D1PhLSHKNLbgwMoR9h
</commit_message>
<xml_diff>
--- a/MetaBorghi_DataTemplate.xlsx
+++ b/MetaBorghi_DataTemplate.xlsx
@@ -117,7 +117,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -139,11 +139,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -179,6 +223,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -586,31 +632,56 @@
           <t>🏢 ANAGRAFICA</t>
         </is>
       </c>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="13" t="n"/>
+      <c r="I1" s="14" t="n"/>
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>📍 LOCALIZZAZIONE</t>
         </is>
       </c>
+      <c r="K1" s="13" t="n"/>
+      <c r="L1" s="13" t="n"/>
+      <c r="M1" s="14" t="n"/>
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>🏷️ TIPOLOGIA</t>
         </is>
       </c>
+      <c r="O1" s="13" t="n"/>
+      <c r="P1" s="13" t="n"/>
+      <c r="Q1" s="13" t="n"/>
+      <c r="R1" s="13" t="n"/>
+      <c r="S1" s="13" t="n"/>
+      <c r="T1" s="14" t="n"/>
       <c r="U1" s="1" t="inlineStr">
         <is>
           <t>📞 CONTATTI</t>
         </is>
       </c>
+      <c r="V1" s="13" t="n"/>
+      <c r="W1" s="13" t="n"/>
+      <c r="X1" s="13" t="n"/>
+      <c r="Y1" s="14" t="n"/>
       <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>🎬 MEDIA</t>
         </is>
       </c>
+      <c r="AA1" s="14" t="n"/>
       <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>🤝 B2B</t>
         </is>
       </c>
+      <c r="AC1" s="13" t="n"/>
+      <c r="AD1" s="13" t="n"/>
+      <c r="AE1" s="14" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -958,433 +1029,1825 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
-      <c r="P4" s="5" t="n"/>
-      <c r="Q4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
-      <c r="S4" s="5" t="n"/>
-      <c r="T4" s="5" t="n"/>
-      <c r="U4" s="5" t="n"/>
-      <c r="V4" s="5" t="n"/>
-      <c r="W4" s="5" t="n"/>
-      <c r="X4" s="5" t="n"/>
-      <c r="Y4" s="5" t="n"/>
-      <c r="Z4" s="5" t="n"/>
-      <c r="AA4" s="5" t="n"/>
-      <c r="AB4" s="5" t="n"/>
-      <c r="AC4" s="5" t="n"/>
-      <c r="AD4" s="5" t="n"/>
-      <c r="AE4" s="5" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>deleo-carni</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>deleo-carni</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>De Leo Carni</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>De Leo Carni S.r.l.</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>IT02345678901</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>1968</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Antonio De Leo</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Ogni salume racconta la storia della nostra terra e del nostro lavoro.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>nusco</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Via Roma 45, 83051 Nusco (AV)</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>40.888</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>La tradizione norcina dell'Alta Irpinia</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>Salumi artigianali irpini prodotti secondo le antiche ricette di famiglia.</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>Da oltre tre generazioni, De Leo Carni custodisce i segreti della norcineria irpina. Ogni salume nasce dalla selezione accurata delle carni di suini allevati allo stato semibrado nelle colline dell'Alta Irpinia, nutrendosi di ghiande e castagne. La lavorazione avviene ancora a mano, con la stagionatura naturale nelle cantine in tufo che garantiscono il microclima perfetto per esaltare i sapori autentici del territorio.</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>BIO, Slow Food</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>2023 - Miglior Soppressata d'Italia - Slow Food</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>PREMIUM</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>info@deleocarni.com</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 64521</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.deleocarni.com</t>
+        </is>
+      </c>
+      <c r="X4" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Z4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/embed/dQw4w9WgXcQ</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/embed?pb=!4v1700000000000!6m8!1m7!1sCAoSLEFGMVFpcE5fX0JQX3RhbWVfY2FrRXdJOXJIeHFYVWNZb2JtVXdMbTBw!2m2!1d40.888!2d15.090!3f0!4f0!5f0.7820865974627469</t>
+        </is>
+      </c>
+      <c r="AB4" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC4" s="5" t="inlineStr">
+        <is>
+          <t>Distribuzione, Ristorazione, Gift box</t>
+        </is>
+      </c>
+      <c r="AD4" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE4" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
-      <c r="O5" s="5" t="n"/>
-      <c r="P5" s="5" t="n"/>
-      <c r="Q5" s="5" t="n"/>
-      <c r="R5" s="5" t="n"/>
-      <c r="S5" s="5" t="n"/>
-      <c r="T5" s="5" t="n"/>
-      <c r="U5" s="5" t="n"/>
-      <c r="V5" s="5" t="n"/>
-      <c r="W5" s="5" t="n"/>
-      <c r="X5" s="5" t="n"/>
-      <c r="Y5" s="5" t="n"/>
-      <c r="Z5" s="5" t="n"/>
-      <c r="AA5" s="5" t="n"/>
-      <c r="AB5" s="5" t="n"/>
-      <c r="AC5" s="5" t="n"/>
-      <c r="AD5" s="5" t="n"/>
-      <c r="AE5" s="5" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>contedoro</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>contedoro</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Conte d'Oro</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Conte d'Oro S.a.s.</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>IT03456789012</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>1952</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Maria Conte</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>L'olio buono si fa in campo, non in frantoio. Il frantoio lo completa.</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>guardia-dei-lombardi</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Contrada Oliveto 12, 83040 Guardia dei Lombardi (AV)</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>40.957</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>15.198</v>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>L'oro verde dell'Irpinia</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>Olio extravergine d'oliva DOP dalle colline irpine.</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Conte d'Oro è un frantoio familiare che produce olio extravergine d'oliva dalle cultivar autoctone dell'Irpinia: Ravece, Ogliarola e Marinese. Gli uliveti si estendono sulle colline di Guardia dei Lombardi, dove il clima e l'altitudine conferiscono all'olio note fruttate intense e un retrogusto leggermente piccante. La molitura avviene entro 24 ore dalla raccolta, a freddo, per preservare ogni proprietà organolettica.</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>DOP, BIO</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>2024 - Gran Menzione Olio DOP - Ercole Olivario</t>
+        </is>
+      </c>
+      <c r="T5" s="5" t="inlineStr">
+        <is>
+          <t>PREMIUM</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>info@contedoro.com</t>
+        </is>
+      </c>
+      <c r="V5" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 41023</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="inlineStr">
+        <is>
+          <t>https://contedoro.com</t>
+        </is>
+      </c>
+      <c r="X5" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y5" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Z5" s="5" t="inlineStr"/>
+      <c r="AA5" s="5" t="inlineStr"/>
+      <c r="AB5" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC5" s="5" t="inlineStr">
+        <is>
+          <t>Export, Ristorazione, Co-branding</t>
+        </is>
+      </c>
+      <c r="AD5" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE5" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
-      <c r="P6" s="5" t="n"/>
-      <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
-      <c r="S6" s="5" t="n"/>
-      <c r="T6" s="5" t="n"/>
-      <c r="U6" s="5" t="n"/>
-      <c r="V6" s="5" t="n"/>
-      <c r="W6" s="5" t="n"/>
-      <c r="X6" s="5" t="n"/>
-      <c r="Y6" s="5" t="n"/>
-      <c r="Z6" s="5" t="n"/>
-      <c r="AA6" s="5" t="n"/>
-      <c r="AB6" s="5" t="n"/>
-      <c r="AC6" s="5" t="n"/>
-      <c r="AD6" s="5" t="n"/>
-      <c r="AE6" s="5" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>boccella-rosa</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>boccella-rosa</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Boccella Rosa</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Boccella Rosa Azienda Vinicola</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>IT04567890123</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Giovanni Boccella</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Il Taurasi è un vino che ha bisogno di tempo. Come le cose migliori.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>castelfranci</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Contrada Vigne 8, 83040 Castelfranci (AV)</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>40.93</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>15.04</v>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>Vini d'Irpinia, anima di vulcano</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>Vini irpini d'eccellenza: Taurasi, Fiano e Greco di Tufo.</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>Boccella Rosa nasce dalla passione di una famiglia di viticoltori che da generazioni coltiva i vitigni autoctoni dell'Irpinia. I vigneti di Aglianico, Fiano e Greco crescono su terreni vulcanici a 500 metri di altitudine, dove le escursioni termiche e i venti montani regalano uve di straordinaria intensità. La vinificazione rispetta i ritmi naturali, con lunghi affinamenti in botti di rovere e in bottiglia.</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>DOCG, DOC, BIO</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>2024 - Tre Bicchieri - Gambero Rosso | 2023 - 95 punti Taurasi Riserva - Wine Spectator</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>PLATINUM</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>info@boccellarosa.it</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 72145</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr">
+        <is>
+          <t>https://boccellarosa.it</t>
+        </is>
+      </c>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y6" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/embed/dQw4w9WgXcQ</t>
+        </is>
+      </c>
+      <c r="AA6" s="5" t="inlineStr"/>
+      <c r="AB6" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC6" s="5" t="inlineStr">
+        <is>
+          <t>Export, Distribuzione, Enoteca, Ristorazione</t>
+        </is>
+      </c>
+      <c r="AD6" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE6" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
-      <c r="P7" s="5" t="n"/>
-      <c r="Q7" s="5" t="n"/>
-      <c r="R7" s="5" t="n"/>
-      <c r="S7" s="5" t="n"/>
-      <c r="T7" s="5" t="n"/>
-      <c r="U7" s="5" t="n"/>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="5" t="n"/>
-      <c r="X7" s="5" t="n"/>
-      <c r="Y7" s="5" t="n"/>
-      <c r="Z7" s="5" t="n"/>
-      <c r="AA7" s="5" t="n"/>
-      <c r="AB7" s="5" t="n"/>
-      <c r="AC7" s="5" t="n"/>
-      <c r="AD7" s="5" t="n"/>
-      <c r="AE7" s="5" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>re-del-bosco</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>re-del-bosco</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Re del Bosco</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Re del Bosco S.r.l.</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>IT05678901234</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Luigi Montella</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Ogni castagna porta con sé il profumo del bosco e la pazienza dei nostri nonni.</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>montella</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Via dei Castagneti 22, 83048 Montella (AV)</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>40.843</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>15.017</v>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>Le castagne più pregiate d'Italia</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>Castagna di Montella IGP e derivati dal cuore dei Picentini.</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>Re del Bosco raccoglie e trasforma la Castagna di Montella IGP, una delle eccellenze più riconosciute della Campania. I castagneti secolari dei Monti Picentini, tra Montella e Bagnoli Irpino, producono frutti di dimensioni generose e sapore dolcissimo. Dall'essiccatura tradizionale nei "gratali" alla farina di castagne macinata a pietra, ogni prodotto preserva il gusto autentico del bosco irpino.</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>IGP, BIO</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>2024 - Premio Eccellenza IGP - Qualivita</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>PREMIUM</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>info@redelbosco.it</t>
+        </is>
+      </c>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 61234</t>
+        </is>
+      </c>
+      <c r="W7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.redelbosco.it</t>
+        </is>
+      </c>
+      <c r="X7" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Z7" s="5" t="inlineStr"/>
+      <c r="AA7" s="5" t="inlineStr"/>
+      <c r="AB7" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC7" s="5" t="inlineStr">
+        <is>
+          <t>Distribuzione, Pasticceria, Export</t>
+        </is>
+      </c>
+      <c r="AD7" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE7" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="5" t="n"/>
-      <c r="P8" s="5" t="n"/>
-      <c r="Q8" s="5" t="n"/>
-      <c r="R8" s="5" t="n"/>
-      <c r="S8" s="5" t="n"/>
-      <c r="T8" s="5" t="n"/>
-      <c r="U8" s="5" t="n"/>
-      <c r="V8" s="5" t="n"/>
-      <c r="W8" s="5" t="n"/>
-      <c r="X8" s="5" t="n"/>
-      <c r="Y8" s="5" t="n"/>
-      <c r="Z8" s="5" t="n"/>
-      <c r="AA8" s="5" t="n"/>
-      <c r="AB8" s="5" t="n"/>
-      <c r="AC8" s="5" t="n"/>
-      <c r="AD8" s="5" t="n"/>
-      <c r="AE8" s="5" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>serrocroce</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>serrocroce</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Serrocroce</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Serrocroce Azienda Agricola</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>IT06789012345</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>2005</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Marco Serra</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Il vino naturale non si fa, si lascia fare. Noi ascoltiamo la vigna.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>castelfranci</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Contrada Serrocroce, 83040 Castelfranci (AV)</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>40.935</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>15.045</v>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Vini naturali dall'Alta Irpinia</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>Vini naturali biodinamici da vigneti d'alta quota.</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>Serrocroce è una cantina boutique che pratica viticoltura biodinamica sui terreni vulcanici dell'Alta Irpinia. I vigneti, coltivati a 600 metri sul livello del mare, producono vini di grande personalità: minerali, freschi, con una complessità aromatica che racconta il territorio. La cantina è scavata nel tufo, dove i vini riposano in anfore di terracotta e botti di castagno locale.</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>BIO, DOC</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>2024 - Vino Naturale dell'Anno - Guida Slow Wine</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>info@serrocroce.it</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 72098</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.serrocroce.it</t>
+        </is>
+      </c>
+      <c r="X8" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y8" s="5" t="inlineStr"/>
+      <c r="Z8" s="5" t="inlineStr"/>
+      <c r="AA8" s="5" t="inlineStr"/>
+      <c r="AB8" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC8" s="5" t="inlineStr">
+        <is>
+          <t>Enoteca, Ristorazione, Export</t>
+        </is>
+      </c>
+      <c r="AD8" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE8" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
-      <c r="N9" s="5" t="n"/>
-      <c r="O9" s="5" t="n"/>
-      <c r="P9" s="5" t="n"/>
-      <c r="Q9" s="5" t="n"/>
-      <c r="R9" s="5" t="n"/>
-      <c r="S9" s="5" t="n"/>
-      <c r="T9" s="5" t="n"/>
-      <c r="U9" s="5" t="n"/>
-      <c r="V9" s="5" t="n"/>
-      <c r="W9" s="5" t="n"/>
-      <c r="X9" s="5" t="n"/>
-      <c r="Y9" s="5" t="n"/>
-      <c r="Z9" s="5" t="n"/>
-      <c r="AA9" s="5" t="n"/>
-      <c r="AB9" s="5" t="n"/>
-      <c r="AC9" s="5" t="n"/>
-      <c r="AD9" s="5" t="n"/>
-      <c r="AE9" s="5" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>caciocavalleria</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>caciocavalleria</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Caciocavalleria De D.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Caciocavalleria De D. S.a.s.</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>IT07890123456</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>1975</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Paolo De Dominicis</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Le nostre vacche Podoliche camminano libere. Il formaggio che producono non ha eguali.</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>lacedonia</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Contrada Masseria 5, 83046 Lacedonia (AV)</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>41.05</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>Il re dei formaggi irpini</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>Caciocavallo Podolico e formaggi di latte crudo dall'Irpinia.</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>La Caciocavalleria De D. è un caseificio artigianale specializzato nella produzione di Caciocavallo Podolico, ottenuto dal latte delle vacche Podoliche allevate al pascolo brado sui pascoli dell'Alta Irpinia. Questo formaggio raro, prodotto solo con latte di razza autoctona, viene stagionato per un minimo di 12 mesi nelle grotte naturali. Il risultato è un formaggio dal gusto intenso, leggermente piccante, con sentori di erbe selvatiche.</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>Slow Food, De.Co.</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>2023 - Presidio Slow Food - Slow Food Italia</t>
+        </is>
+      </c>
+      <c r="T9" s="5" t="inlineStr">
+        <is>
+          <t>PREMIUM</t>
+        </is>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>info@caciocavalleriaded.it</t>
+        </is>
+      </c>
+      <c r="V9" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 85012</t>
+        </is>
+      </c>
+      <c r="W9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.caciocavalleriaded.it</t>
+        </is>
+      </c>
+      <c r="X9" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y9" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Z9" s="5" t="inlineStr"/>
+      <c r="AA9" s="5" t="inlineStr"/>
+      <c r="AB9" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC9" s="5" t="inlineStr">
+        <is>
+          <t>Distribuzione, Ristorazione, Export</t>
+        </is>
+      </c>
+      <c r="AD9" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE9" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="5" t="n"/>
-      <c r="O10" s="5" t="n"/>
-      <c r="P10" s="5" t="n"/>
-      <c r="Q10" s="5" t="n"/>
-      <c r="R10" s="5" t="n"/>
-      <c r="S10" s="5" t="n"/>
-      <c r="T10" s="5" t="n"/>
-      <c r="U10" s="5" t="n"/>
-      <c r="V10" s="5" t="n"/>
-      <c r="W10" s="5" t="n"/>
-      <c r="X10" s="5" t="n"/>
-      <c r="Y10" s="5" t="n"/>
-      <c r="Z10" s="5" t="n"/>
-      <c r="AA10" s="5" t="n"/>
-      <c r="AB10" s="5" t="n"/>
-      <c r="AC10" s="5" t="n"/>
-      <c r="AD10" s="5" t="n"/>
-      <c r="AE10" s="5" t="n"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>carmasciando</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>carmasciando</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Carmasciando</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Carmasciando Azienda Agricola</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>IT08901234567</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>2010</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Salvatore Carmasciando</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Il vino è solo l'inizio. Venite a vivere questa terra.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>torella-dei-lombardi</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Contrada Piano 15, 83057 Torella dei Lombardi (AV)</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>40.94</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>15.113</v>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>MISTO</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>Vino, terra, accoglienza</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>Cantina con agriturismo e esperienze nel cuore dell'Irpinia.</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>Carmasciando è un progetto di vita che unisce viticoltura, ospitalità e cultura del territorio. La cantina produce vini da vitigni autoctoni irpini, mentre l'agriturismo offre esperienze immersive: dalle vendemmie partecipate alle cene in vigna, dalla raccolta delle olive ai laboratori di cucina irpina. Un luogo dove il tempo rallenta e i sapori raccontano storie.</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>BIO, DOC</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr"/>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>PLATINUM</t>
+        </is>
+      </c>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>info@carmasciando.it</t>
+        </is>
+      </c>
+      <c r="V10" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 49876</t>
+        </is>
+      </c>
+      <c r="W10" s="5" t="inlineStr">
+        <is>
+          <t>https://carmasciando.it</t>
+        </is>
+      </c>
+      <c r="X10" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y10" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Z10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/embed/dQw4w9WgXcQ</t>
+        </is>
+      </c>
+      <c r="AA10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/embed?pb=!4v1700000000000!6m8!1m7!1sCAoSLEFGMVFpcE5fX0JQX3RhbWVfY2FrRXdJOXJIeHFYVWNZb2JtVXdMbTBw!2m2!1d40.940!2d15.113!3f0!4f0!5f0.7820865974627469</t>
+        </is>
+      </c>
+      <c r="AB10" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC10" s="5" t="inlineStr">
+        <is>
+          <t>Turismo, Ristorazione, Eventi, Co-branding</t>
+        </is>
+      </c>
+      <c r="AD10" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE10" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
-      <c r="N11" s="5" t="n"/>
-      <c r="O11" s="5" t="n"/>
-      <c r="P11" s="5" t="n"/>
-      <c r="Q11" s="5" t="n"/>
-      <c r="R11" s="5" t="n"/>
-      <c r="S11" s="5" t="n"/>
-      <c r="T11" s="5" t="n"/>
-      <c r="U11" s="5" t="n"/>
-      <c r="V11" s="5" t="n"/>
-      <c r="W11" s="5" t="n"/>
-      <c r="X11" s="5" t="n"/>
-      <c r="Y11" s="5" t="n"/>
-      <c r="Z11" s="5" t="n"/>
-      <c r="AA11" s="5" t="n"/>
-      <c r="AB11" s="5" t="n"/>
-      <c r="AC11" s="5" t="n"/>
-      <c r="AD11" s="5" t="n"/>
-      <c r="AE11" s="5" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>torronificio-del-casale</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>torronificio-del-casale</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Torronificio del Casale</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Torronificio del Casale S.r.l.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>IT09012345678</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>1890</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Rosa Del Casale</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Il segreto del nostro torrone? Il tempo. Non abbiamo mai avuto fretta.</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>sant-angelo-dei-lombardi</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Via Mancini 8, 83054 Sant'Angelo dei Lombardi (AV)</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>40.927</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>15.175</v>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>L'arte del torrone dal 1890</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>Torroni artigianali irpini: miele, nocciole e tradizione.</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>Il Torronificio del Casale porta avanti una tradizione dolciaria che risale alla fine dell'Ottocento. Il torrone viene prodotto con miele di castagno dell'Irpinia, nocciole Tonde di Giffoni e mandorle selezionate, seguendo il metodo di cottura lenta in caldaie di rame. Ogni barretta è confezionata a mano, come si faceva un tempo. Una dolcezza autentica che racconta la storia del Natale irpino.</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>De.Co., Slow Food</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>2024 - Eccellenza Artigiana - CNA Campania</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>PREMIUM</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>info@torronificiodelcasale.com</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 23456</t>
+        </is>
+      </c>
+      <c r="W11" s="5" t="inlineStr">
+        <is>
+          <t>https://www.torronificiodelcasale.com</t>
+        </is>
+      </c>
+      <c r="X11" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y11" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Z11" s="5" t="inlineStr"/>
+      <c r="AA11" s="5" t="inlineStr"/>
+      <c r="AB11" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC11" s="5" t="inlineStr">
+        <is>
+          <t>Distribuzione, Gift box, Export, HoReCa</t>
+        </is>
+      </c>
+      <c r="AD11" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE11" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
-      <c r="K12" s="5" t="n"/>
-      <c r="L12" s="5" t="n"/>
-      <c r="M12" s="5" t="n"/>
-      <c r="N12" s="5" t="n"/>
-      <c r="O12" s="5" t="n"/>
-      <c r="P12" s="5" t="n"/>
-      <c r="Q12" s="5" t="n"/>
-      <c r="R12" s="5" t="n"/>
-      <c r="S12" s="5" t="n"/>
-      <c r="T12" s="5" t="n"/>
-      <c r="U12" s="5" t="n"/>
-      <c r="V12" s="5" t="n"/>
-      <c r="W12" s="5" t="n"/>
-      <c r="X12" s="5" t="n"/>
-      <c r="Y12" s="5" t="n"/>
-      <c r="Z12" s="5" t="n"/>
-      <c r="AA12" s="5" t="n"/>
-      <c r="AB12" s="5" t="n"/>
-      <c r="AC12" s="5" t="n"/>
-      <c r="AD12" s="5" t="n"/>
-      <c r="AE12" s="5" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>dolci-terre</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>dolci-terre</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Dolci Terre</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Dolci Terre di Irpinia</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>IT10123456789</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>2008</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Francesca Iannaccone</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>La natura ci regala tutto. Noi lo mettiamo in un vasetto.</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>montella</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Via Fontana 30, 83048 Montella (AV)</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>40.845</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>15.02</v>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>La dolcezza autentica dell'Irpinia</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>Confetture, mieli e conserve dal cuore verde dell'Irpinia.</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>Dolci Terre trasforma i frutti spontanei e coltivati dell'Alta Irpinia in confetture, mieli aromatici e conserve. Dalle fichi tardive ai pomodori secchi, dal miele di castagno a quello millefiori di montagna: ogni vasetto è il risultato di una filiera cortissima, dalla pianta al prodotto finito in meno di 48 ore. Senza conservanti, senza coloranti, solo il sapore vero della terra.</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>BIO</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr"/>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>info@dolciterre.it</t>
+        </is>
+      </c>
+      <c r="V12" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 61890</t>
+        </is>
+      </c>
+      <c r="W12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.dolciterre.it</t>
+        </is>
+      </c>
+      <c r="X12" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y12" s="5" t="inlineStr"/>
+      <c r="Z12" s="5" t="inlineStr"/>
+      <c r="AA12" s="5" t="inlineStr"/>
+      <c r="AB12" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AC12" s="5" t="inlineStr"/>
+      <c r="AD12" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE12" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
-      <c r="L13" s="5" t="n"/>
-      <c r="M13" s="5" t="n"/>
-      <c r="N13" s="5" t="n"/>
-      <c r="O13" s="5" t="n"/>
-      <c r="P13" s="5" t="n"/>
-      <c r="Q13" s="5" t="n"/>
-      <c r="R13" s="5" t="n"/>
-      <c r="S13" s="5" t="n"/>
-      <c r="T13" s="5" t="n"/>
-      <c r="U13" s="5" t="n"/>
-      <c r="V13" s="5" t="n"/>
-      <c r="W13" s="5" t="n"/>
-      <c r="X13" s="5" t="n"/>
-      <c r="Y13" s="5" t="n"/>
-      <c r="Z13" s="5" t="n"/>
-      <c r="AA13" s="5" t="n"/>
-      <c r="AB13" s="5" t="n"/>
-      <c r="AC13" s="5" t="n"/>
-      <c r="AD13" s="5" t="n"/>
-      <c r="AE13" s="5" t="n"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>tenuta-pepe</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>tenuta-pepe</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Tenuta Pepe</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Tenuta Pepe S.a.s.</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>IT11234567890</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>1986</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Roberto Pepe</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>L'Irpinia è la Borgogna del Sud. I nostri vini lo dimostrano.</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>lioni</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Contrada Vigne 5, 83047 Lioni (AV)</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>40.878</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>15.183</v>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>Tradizione vinicola dal 1986</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>Vini d'autore dall'Irpinia: Taurasi DOCG e Fiano di Avellino.</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>Tenuta Pepe è una delle cantine storiche dell'Irpinia, fondata nel 1986 dalla famiglia Pepe con l'obiettivo di valorizzare i grandi vitigni autoctoni campani. I vigneti si estendono su 15 ettari di terreni argilloso-calcarei, ideali per l'Aglianico e il Fiano. La cantina combina metodi tradizionali con tecnologia enologica moderna, producendo vini eleganti che esprimono il terroir irpino.</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>DOCG, DOC, BIO</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>2024 - Tre Bicchieri Taurasi - Gambero Rosso | 2023 - 93 punti Fiano - James Suckling</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>PLATINUM</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>info@tenutapepe.it</t>
+        </is>
+      </c>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 42567</t>
+        </is>
+      </c>
+      <c r="W13" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tenutapepe.it</t>
+        </is>
+      </c>
+      <c r="X13" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y13" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Z13" s="5" t="inlineStr"/>
+      <c r="AA13" s="5" t="inlineStr"/>
+      <c r="AB13" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC13" s="5" t="inlineStr">
+        <is>
+          <t>Export, Enoteca, Ristorazione, Hotel</t>
+        </is>
+      </c>
+      <c r="AD13" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE13" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="n"/>
-      <c r="L14" s="5" t="n"/>
-      <c r="M14" s="5" t="n"/>
-      <c r="N14" s="5" t="n"/>
-      <c r="O14" s="5" t="n"/>
-      <c r="P14" s="5" t="n"/>
-      <c r="Q14" s="5" t="n"/>
-      <c r="R14" s="5" t="n"/>
-      <c r="S14" s="5" t="n"/>
-      <c r="T14" s="5" t="n"/>
-      <c r="U14" s="5" t="n"/>
-      <c r="V14" s="5" t="n"/>
-      <c r="W14" s="5" t="n"/>
-      <c r="X14" s="5" t="n"/>
-      <c r="Y14" s="5" t="n"/>
-      <c r="Z14" s="5" t="n"/>
-      <c r="AA14" s="5" t="n"/>
-      <c r="AB14" s="5" t="n"/>
-      <c r="AC14" s="5" t="n"/>
-      <c r="AD14" s="5" t="n"/>
-      <c r="AE14" s="5" t="n"/>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>sella-delle-spine</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>sella-delle-spine</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Sella delle Spine</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Sella delle Spine Azienda Agricola</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>IT12345678901</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>1998</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Anna Spinelli</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Il Greco di Tufo è la voce della terra vulcanica. Noi lo lasciamo parlare.</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>calitri</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Contrada Spine 3, 83045 Calitri (AV)</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="M14" s="5" t="n">
+        <v>15.44</v>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Dove nasce il Greco di Tufo</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>Greco di Tufo DOCG e bianchi d'alta quota.</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Sella delle Spine è una piccola cantina familiare che coltiva Greco di Tufo sui pendii vulcanici dell'Irpinia. I vigneti, esposti a sud-est, beneficiano delle brezze montane e delle escursioni termiche che conferiscono al Greco una freschezza e una mineralità uniche. La produzione è volutamente limitata per garantire la massima qualità in ogni bottiglia.</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr">
+        <is>
+          <t>DOCG, BIO</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="inlineStr"/>
+      <c r="T14" s="5" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>info@selladellespine.com</t>
+        </is>
+      </c>
+      <c r="V14" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 35012</t>
+        </is>
+      </c>
+      <c r="W14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.selladellespine.com</t>
+        </is>
+      </c>
+      <c r="X14" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y14" s="5" t="inlineStr"/>
+      <c r="Z14" s="5" t="inlineStr"/>
+      <c r="AA14" s="5" t="inlineStr"/>
+      <c r="AB14" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC14" s="5" t="inlineStr">
+        <is>
+          <t>Enoteca, Export</t>
+        </is>
+      </c>
+      <c r="AD14" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE14" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
-      <c r="L15" s="5" t="n"/>
-      <c r="M15" s="5" t="n"/>
-      <c r="N15" s="5" t="n"/>
-      <c r="O15" s="5" t="n"/>
-      <c r="P15" s="5" t="n"/>
-      <c r="Q15" s="5" t="n"/>
-      <c r="R15" s="5" t="n"/>
-      <c r="S15" s="5" t="n"/>
-      <c r="T15" s="5" t="n"/>
-      <c r="U15" s="5" t="n"/>
-      <c r="V15" s="5" t="n"/>
-      <c r="W15" s="5" t="n"/>
-      <c r="X15" s="5" t="n"/>
-      <c r="Y15" s="5" t="n"/>
-      <c r="Z15" s="5" t="n"/>
-      <c r="AA15" s="5" t="n"/>
-      <c r="AB15" s="5" t="n"/>
-      <c r="AC15" s="5" t="n"/>
-      <c r="AD15" s="5" t="n"/>
-      <c r="AE15" s="5" t="n"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>bifulco</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>bifulco</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Bifulco</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Bifulco Alimentari S.r.l.</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>IT13456789012</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>1972</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Carlo Bifulco</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>La pasta buona si riconosce dal profumo del grano, non dall'etichetta.</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>lioni</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Via Industria 18, 83047 Lioni (AV)</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>40.88</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>15.185</v>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>PRODUTTORE_FOOD</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>Pasta e tradizione irpina</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Pasta artigianale e prodotti da forno della tradizione irpina.</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Bifulco è un pastificio artigianale che produce pasta di semola di grano duro con trafilatura al bronzo e essiccazione lenta. I fusilli al ferretto, i cavatelli e le lagane sono le specialità della casa, preparate con lo stesso metodo che le massaie irpine usano da secoli. Il grano proviene dalle campagne dell'Alta Irpinia, macinato in piccoli mulini locali.</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>De.Co.</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr"/>
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="U15" s="5" t="inlineStr">
+        <is>
+          <t>info@bifulco.it</t>
+        </is>
+      </c>
+      <c r="V15" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 42890</t>
+        </is>
+      </c>
+      <c r="W15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bifulco.it</t>
+        </is>
+      </c>
+      <c r="X15" s="5" t="inlineStr"/>
+      <c r="Y15" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Z15" s="5" t="inlineStr"/>
+      <c r="AA15" s="5" t="inlineStr"/>
+      <c r="AB15" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC15" s="5" t="inlineStr">
+        <is>
+          <t>Distribuzione, Ristorazione</t>
+        </is>
+      </c>
+      <c r="AD15" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE15" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
-      <c r="L16" s="5" t="n"/>
-      <c r="M16" s="5" t="n"/>
-      <c r="N16" s="5" t="n"/>
-      <c r="O16" s="5" t="n"/>
-      <c r="P16" s="5" t="n"/>
-      <c r="Q16" s="5" t="n"/>
-      <c r="R16" s="5" t="n"/>
-      <c r="S16" s="5" t="n"/>
-      <c r="T16" s="5" t="n"/>
-      <c r="U16" s="5" t="n"/>
-      <c r="V16" s="5" t="n"/>
-      <c r="W16" s="5" t="n"/>
-      <c r="X16" s="5" t="n"/>
-      <c r="Y16" s="5" t="n"/>
-      <c r="Z16" s="5" t="n"/>
-      <c r="AA16" s="5" t="n"/>
-      <c r="AB16" s="5" t="n"/>
-      <c r="AC16" s="5" t="n"/>
-      <c r="AD16" s="5" t="n"/>
-      <c r="AE16" s="5" t="n"/>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>akudunniad</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>akudunniad</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>A' Ku Dunniad</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>A' Ku Dunniad Cooperativa Sociale</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>IT14567890123</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>2015</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Teresa Calitri</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Restare è la forma più coraggiosa di innovazione.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>calitri</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Via del Borgo 7, 83045 Calitri (AV)</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="n">
+        <v>40.895</v>
+      </c>
+      <c r="M16" s="5" t="n">
+        <v>15.435</v>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>MISTO</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Il sapore della comunità</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>Cooperativa sociale: prodotti tipici, ospitalità e inclusione.</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>A' Ku Dunniad (dal dialetto irpino "come una volta") è una cooperativa sociale che unisce produzione agroalimentare, turismo responsabile e inclusione sociale. I prodotti — conserve, confetture, pasta fresca — nascono dal lavoro di una comunità che ha scelto di restare e innovare nei borghi dell'Alta Irpinia. Un modello di economia circolare e sostenibile.</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>BIO</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>2023 - Premio Innovazione Sociale - Ashoka Italia</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>PREMIUM</t>
+        </is>
+      </c>
+      <c r="U16" s="5" t="inlineStr">
+        <is>
+          <t>info@akudunniad.it</t>
+        </is>
+      </c>
+      <c r="V16" s="5" t="inlineStr">
+        <is>
+          <t>+39 0827 35890</t>
+        </is>
+      </c>
+      <c r="W16" s="5" t="inlineStr">
+        <is>
+          <t>https://akudunniad.it</t>
+        </is>
+      </c>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Y16" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="Z16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/embed/dQw4w9WgXcQ</t>
+        </is>
+      </c>
+      <c r="AA16" s="5" t="inlineStr"/>
+      <c r="AB16" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC16" s="5" t="inlineStr">
+        <is>
+          <t>Turismo, Inclusione sociale, Distribuzione</t>
+        </is>
+      </c>
+      <c r="AD16" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE16" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="5" t="n"/>
@@ -2676,31 +4139,63 @@
           <t>🎯 ANAGRAFICA</t>
         </is>
       </c>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="14" t="n"/>
       <c r="H1" s="6" t="inlineStr">
         <is>
           <t>📝 DESCRIZIONI</t>
         </is>
       </c>
+      <c r="I1" s="14" t="n"/>
       <c r="J1" s="6" t="inlineStr">
         <is>
           <t>⚙️ DETTAGLI</t>
         </is>
       </c>
+      <c r="K1" s="13" t="n"/>
+      <c r="L1" s="13" t="n"/>
+      <c r="M1" s="13" t="n"/>
+      <c r="N1" s="13" t="n"/>
+      <c r="O1" s="14" t="n"/>
       <c r="P1" s="6" t="inlineStr">
         <is>
           <t>✅ INCLUDE / ESCLUDE</t>
         </is>
       </c>
+      <c r="Q1" s="13" t="n"/>
+      <c r="R1" s="13" t="n"/>
+      <c r="S1" s="13" t="n"/>
+      <c r="T1" s="13" t="n"/>
+      <c r="U1" s="14" t="n"/>
       <c r="V1" s="6" t="inlineStr">
         <is>
           <t>📍 LOCALIZZAZIONE</t>
         </is>
       </c>
+      <c r="W1" s="14" t="n"/>
       <c r="X1" s="6" t="inlineStr">
         <is>
           <t>🕐 PROGRAMMA</t>
         </is>
       </c>
+      <c r="Y1" s="13" t="n"/>
+      <c r="Z1" s="13" t="n"/>
+      <c r="AA1" s="13" t="n"/>
+      <c r="AB1" s="13" t="n"/>
+      <c r="AC1" s="13" t="n"/>
+      <c r="AD1" s="13" t="n"/>
+      <c r="AE1" s="13" t="n"/>
+      <c r="AF1" s="13" t="n"/>
+      <c r="AG1" s="13" t="n"/>
+      <c r="AH1" s="13" t="n"/>
+      <c r="AI1" s="13" t="n"/>
+      <c r="AJ1" s="13" t="n"/>
+      <c r="AK1" s="13" t="n"/>
+      <c r="AL1" s="14" t="n"/>
       <c r="AM1" s="6" t="inlineStr">
         <is>
           <t>📊 STATO</t>
@@ -5182,9 +6677,9 @@
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="X1:AL1"/>
+    <mergeCell ref="AM1"/>
+    <mergeCell ref="P1:U1"/>
     <mergeCell ref="J1:O1"/>
-    <mergeCell ref="P1:U1"/>
-    <mergeCell ref="AM1"/>
     <mergeCell ref="V1:W1"/>
     <mergeCell ref="H1:I1"/>
   </mergeCells>
@@ -5239,26 +6734,50 @@
           <t>🎨 ANAGRAFICA</t>
         </is>
       </c>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="14" t="n"/>
       <c r="F1" s="7" t="inlineStr">
         <is>
           <t>📝 DESCRIZIONI</t>
         </is>
       </c>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="13" t="n"/>
+      <c r="I1" s="14" t="n"/>
       <c r="J1" s="7" t="inlineStr">
         <is>
           <t>📐 SPECIFICHE</t>
         </is>
       </c>
+      <c r="K1" s="13" t="n"/>
+      <c r="L1" s="13" t="n"/>
+      <c r="M1" s="13" t="n"/>
+      <c r="N1" s="13" t="n"/>
+      <c r="O1" s="13" t="n"/>
+      <c r="P1" s="13" t="n"/>
+      <c r="Q1" s="14" t="n"/>
       <c r="R1" s="7" t="inlineStr">
         <is>
           <t>🎛️ PERSONALIZZAZIONI</t>
         </is>
       </c>
+      <c r="S1" s="13" t="n"/>
+      <c r="T1" s="13" t="n"/>
+      <c r="U1" s="13" t="n"/>
+      <c r="V1" s="13" t="n"/>
+      <c r="W1" s="14" t="n"/>
       <c r="X1" s="7" t="inlineStr">
         <is>
           <t>🔄 PROCESSO</t>
         </is>
       </c>
+      <c r="Y1" s="13" t="n"/>
+      <c r="Z1" s="13" t="n"/>
+      <c r="AA1" s="13" t="n"/>
+      <c r="AB1" s="13" t="n"/>
+      <c r="AC1" s="14" t="n"/>
       <c r="AD1" s="7" t="inlineStr">
         <is>
           <t>📊 STATO</t>
@@ -7246,26 +8765,45 @@
           <t>🛒 ANAGRAFICA</t>
         </is>
       </c>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="14" t="n"/>
       <c r="G1" s="8" t="inlineStr">
         <is>
           <t>📝 DESCRIZIONI</t>
         </is>
       </c>
+      <c r="H1" s="13" t="n"/>
+      <c r="I1" s="13" t="n"/>
+      <c r="J1" s="14" t="n"/>
       <c r="K1" s="8" t="inlineStr">
         <is>
           <t>📐 SPECIFICHE</t>
         </is>
       </c>
+      <c r="L1" s="13" t="n"/>
+      <c r="M1" s="13" t="n"/>
+      <c r="N1" s="13" t="n"/>
+      <c r="O1" s="13" t="n"/>
+      <c r="P1" s="13" t="n"/>
+      <c r="Q1" s="13" t="n"/>
+      <c r="R1" s="14" t="n"/>
       <c r="S1" s="8" t="inlineStr">
         <is>
           <t>📦 LOGISTICA</t>
         </is>
       </c>
+      <c r="T1" s="13" t="n"/>
+      <c r="U1" s="13" t="n"/>
+      <c r="V1" s="14" t="n"/>
       <c r="W1" s="8" t="inlineStr">
         <is>
           <t>📊 STATO</t>
         </is>
       </c>
+      <c r="X1" s="14" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -8895,41 +10433,64 @@
           <t>🏨 ANAGRAFICA</t>
         </is>
       </c>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="14" t="n"/>
       <c r="G1" s="9" t="inlineStr">
         <is>
           <t>📍 LOCALIZZAZIONE</t>
         </is>
       </c>
+      <c r="H1" s="13" t="n"/>
+      <c r="I1" s="13" t="n"/>
+      <c r="J1" s="14" t="n"/>
       <c r="K1" s="9" t="inlineStr">
         <is>
           <t>📝 DESCRIZIONI</t>
         </is>
       </c>
+      <c r="L1" s="13" t="n"/>
+      <c r="M1" s="14" t="n"/>
       <c r="N1" s="9" t="inlineStr">
         <is>
           <t>⚙️ STRUTTURA</t>
         </is>
       </c>
+      <c r="O1" s="13" t="n"/>
+      <c r="P1" s="13" t="n"/>
+      <c r="Q1" s="13" t="n"/>
+      <c r="R1" s="13" t="n"/>
+      <c r="S1" s="13" t="n"/>
+      <c r="T1" s="14" t="n"/>
       <c r="U1" s="9" t="inlineStr">
         <is>
           <t>✅ SERVIZI</t>
         </is>
       </c>
+      <c r="V1" s="13" t="n"/>
+      <c r="W1" s="13" t="n"/>
+      <c r="X1" s="14" t="n"/>
       <c r="Y1" s="9" t="inlineStr">
         <is>
           <t>📞 PRENOTAZIONI</t>
         </is>
       </c>
+      <c r="Z1" s="13" t="n"/>
+      <c r="AA1" s="14" t="n"/>
       <c r="AB1" s="9" t="inlineStr">
         <is>
           <t>🎬 MEDIA</t>
         </is>
       </c>
+      <c r="AC1" s="14" t="n"/>
       <c r="AD1" s="9" t="inlineStr">
         <is>
           <t>📊 STATO</t>
         </is>
       </c>
+      <c r="AE1" s="14" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -10977,26 +12538,40 @@
           <t>🏘️ IDENTIFICATIVO</t>
         </is>
       </c>
+      <c r="B1" s="14" t="n"/>
       <c r="C1" s="10" t="inlineStr">
         <is>
           <t>📝 CONTENUTO</t>
         </is>
       </c>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="13" t="n"/>
+      <c r="I1" s="14" t="n"/>
       <c r="J1" s="10" t="inlineStr">
         <is>
           <t>📍 DATI GEOGRAFICI</t>
         </is>
       </c>
+      <c r="K1" s="13" t="n"/>
+      <c r="L1" s="13" t="n"/>
+      <c r="M1" s="13" t="n"/>
+      <c r="N1" s="14" t="n"/>
       <c r="O1" s="10" t="inlineStr">
         <is>
           <t>📊 STATISTICHE</t>
         </is>
       </c>
+      <c r="P1" s="13" t="n"/>
+      <c r="Q1" s="14" t="n"/>
       <c r="R1" s="10" t="inlineStr">
         <is>
           <t>🎬 MEDIA</t>
         </is>
       </c>
+      <c r="S1" s="14" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: formato Lacedonia per tutti i borghi — Excel completo + Ristorazione
- Excel: tutti i fogli popolati con 1 esempio Lacedonia (Aziende, Esperienze,
  Artigianato, Prodotti Food, Ospitalità, Borghi)
- Nuovo foglio Ristorazione con header, istruzioni e esempio (Trattoria del Borgo)
- Borghi: macro-descrizione Lacedonia (MAVI, San Gerardo, De Sanctis, etc.)
- Borghi: aggiornati highlights, prodotti (zafferano irpino), esperienze (MAVI, Museo Diocesano)
- BoroughDetailPage: titolo video → "Scopri {nome}", tour → "Passeggia a {nome}. Tour virtuale a 360°"

https://claude.ai/code/session_018oe8D1PhLSHKNLbgwMoR9h
</commit_message>
<xml_diff>
--- a/MetaBorghi_DataTemplate.xlsx
+++ b/MetaBorghi_DataTemplate.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Artigianato" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Prodotti Food" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Ospitalità" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Borghi" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="📋 Legenda" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Ristorazione" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Borghi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="📋 Legenda" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +59,30 @@
     <font>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -116,8 +139,20 @@
         <fgColor rgb="00566573"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -183,11 +218,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -225,6 +274,22 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1029,1825 +1094,541 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>deleo-carni</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>deleo-carni</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>De Leo Carni</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>De Leo Carni S.r.l.</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>IT02345678901</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>1968</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>Antonio De Leo</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>Ogni salume racconta la storia della nostra terra e del nostro lavoro.</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>nusco</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>Via Roma 45, 83051 Nusco (AV)</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="n">
-        <v>40.888</v>
-      </c>
-      <c r="M4" s="5" t="n">
-        <v>15.09</v>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>caciocavalleria</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>caciocavalleria</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Caciocavalleria De D.</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Caciocavalleria De D. S.a.s.</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>IT07890123456</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="n">
+        <v>1975</v>
+      </c>
+      <c r="G4" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Paolo De Dominicis</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>Le nostre vacche Podoliche camminano libere. Il formaggio che producono non ha eguali.</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>lacedonia</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>Contrada Masseria 5, 83046 Lacedonia (AV)</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="n">
+        <v>41.05</v>
+      </c>
+      <c r="M4" s="15" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="N4" s="15" t="inlineStr">
         <is>
           <t>PRODUTTORE_FOOD</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>La tradizione norcina dell'Alta Irpinia</t>
-        </is>
-      </c>
-      <c r="P4" s="5" t="inlineStr">
-        <is>
-          <t>Salumi artigianali irpini prodotti secondo le antiche ricette di famiglia.</t>
-        </is>
-      </c>
-      <c r="Q4" s="5" t="inlineStr">
-        <is>
-          <t>Da oltre tre generazioni, De Leo Carni custodisce i segreti della norcineria irpina. Ogni salume nasce dalla selezione accurata delle carni di suini allevati allo stato semibrado nelle colline dell'Alta Irpinia, nutrendosi di ghiande e castagne. La lavorazione avviene ancora a mano, con la stagionatura naturale nelle cantine in tufo che garantiscono il microclima perfetto per esaltare i sapori autentici del territorio.</t>
-        </is>
-      </c>
-      <c r="R4" s="5" t="inlineStr">
-        <is>
-          <t>BIO, Slow Food</t>
-        </is>
-      </c>
-      <c r="S4" s="5" t="inlineStr">
-        <is>
-          <t>2023 - Miglior Soppressata d'Italia - Slow Food</t>
-        </is>
-      </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="O4" s="15" t="inlineStr">
+        <is>
+          <t>Il re dei formaggi irpini</t>
+        </is>
+      </c>
+      <c r="P4" s="15" t="inlineStr">
+        <is>
+          <t>Caciocavallo Podolico e formaggi di latte crudo dall'Irpinia.</t>
+        </is>
+      </c>
+      <c r="Q4" s="15" t="inlineStr">
+        <is>
+          <t>La Caciocavalleria De D. è un caseificio artigianale specializzato nella produzione di Caciocavallo Podolico, ottenuto dal latte delle vacche Podoliche allevate al pascolo brado sui pascoli dell'Alta Irpinia. Questo formaggio raro, prodotto solo con latte di razza autoctona, viene stagionato per un minimo di 12 mesi nelle grotte naturali. Il risultato è un formaggio dal gusto intenso, leggermente piccante, con sentori di erbe selvatiche.</t>
+        </is>
+      </c>
+      <c r="R4" s="15" t="inlineStr">
+        <is>
+          <t>Slow Food, De.Co.</t>
+        </is>
+      </c>
+      <c r="S4" s="15" t="inlineStr">
+        <is>
+          <t>2023 - Presidio Slow Food - Slow Food Italia</t>
+        </is>
+      </c>
+      <c r="T4" s="15" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
-        <is>
-          <t>info@deleocarni.com</t>
-        </is>
-      </c>
-      <c r="V4" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 64521</t>
-        </is>
-      </c>
-      <c r="W4" s="5" t="inlineStr">
-        <is>
-          <t>https://www.deleocarni.com</t>
-        </is>
-      </c>
-      <c r="X4" s="5" t="inlineStr">
+      <c r="U4" s="15" t="inlineStr">
+        <is>
+          <t>info@caciocavalleriaded.it</t>
+        </is>
+      </c>
+      <c r="V4" s="15" t="inlineStr">
+        <is>
+          <t>+39 0827 85012</t>
+        </is>
+      </c>
+      <c r="W4" s="15" t="inlineStr">
+        <is>
+          <t>https://www.caciocavalleriaded.it</t>
+        </is>
+      </c>
+      <c r="X4" s="15" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="Y4" s="15" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="Z4" s="5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/embed/dQw4w9WgXcQ</t>
-        </is>
-      </c>
-      <c r="AA4" s="5" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/embed?pb=!4v1700000000000!6m8!1m7!1sCAoSLEFGMVFpcE5fX0JQX3RhbWVfY2FrRXdJOXJIeHFYVWNZb2JtVXdMbTBw!2m2!1d40.888!2d15.090!3f0!4f0!5f0.7820865974627469</t>
-        </is>
-      </c>
-      <c r="AB4" s="5" t="inlineStr">
+      <c r="Z4" s="15" t="inlineStr"/>
+      <c r="AA4" s="15" t="inlineStr"/>
+      <c r="AB4" s="15" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="AC4" s="5" t="inlineStr">
-        <is>
-          <t>Distribuzione, Ristorazione, Gift box</t>
-        </is>
-      </c>
-      <c r="AD4" s="5" t="inlineStr">
+      <c r="AC4" s="15" t="inlineStr">
+        <is>
+          <t>Distribuzione, Ristorazione, Export</t>
+        </is>
+      </c>
+      <c r="AD4" s="15" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="AE4" s="5" t="inlineStr">
+      <c r="AE4" s="15" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>contedoro</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>contedoro</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Conte d'Oro</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Conte d'Oro S.a.s.</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>IT03456789012</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>1952</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Maria Conte</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>L'olio buono si fa in campo, non in frantoio. Il frantoio lo completa.</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>guardia-dei-lombardi</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Contrada Oliveto 12, 83040 Guardia dei Lombardi (AV)</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="n">
-        <v>40.957</v>
-      </c>
-      <c r="M5" s="5" t="n">
-        <v>15.198</v>
-      </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>PRODUTTORE_FOOD</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>L'oro verde dell'Irpinia</t>
-        </is>
-      </c>
-      <c r="P5" s="5" t="inlineStr">
-        <is>
-          <t>Olio extravergine d'oliva DOP dalle colline irpine.</t>
-        </is>
-      </c>
-      <c r="Q5" s="5" t="inlineStr">
-        <is>
-          <t>Conte d'Oro è un frantoio familiare che produce olio extravergine d'oliva dalle cultivar autoctone dell'Irpinia: Ravece, Ogliarola e Marinese. Gli uliveti si estendono sulle colline di Guardia dei Lombardi, dove il clima e l'altitudine conferiscono all'olio note fruttate intense e un retrogusto leggermente piccante. La molitura avviene entro 24 ore dalla raccolta, a freddo, per preservare ogni proprietà organolettica.</t>
-        </is>
-      </c>
-      <c r="R5" s="5" t="inlineStr">
-        <is>
-          <t>DOP, BIO</t>
-        </is>
-      </c>
-      <c r="S5" s="5" t="inlineStr">
-        <is>
-          <t>2024 - Gran Menzione Olio DOP - Ercole Olivario</t>
-        </is>
-      </c>
-      <c r="T5" s="5" t="inlineStr">
-        <is>
-          <t>PREMIUM</t>
-        </is>
-      </c>
-      <c r="U5" s="5" t="inlineStr">
-        <is>
-          <t>info@contedoro.com</t>
-        </is>
-      </c>
-      <c r="V5" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 41023</t>
-        </is>
-      </c>
-      <c r="W5" s="5" t="inlineStr">
-        <is>
-          <t>https://contedoro.com</t>
-        </is>
-      </c>
-      <c r="X5" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y5" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Z5" s="5" t="inlineStr"/>
-      <c r="AA5" s="5" t="inlineStr"/>
-      <c r="AB5" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC5" s="5" t="inlineStr">
-        <is>
-          <t>Export, Ristorazione, Co-branding</t>
-        </is>
-      </c>
-      <c r="AD5" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE5" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="5" t="n"/>
+      <c r="N5" s="5" t="n"/>
+      <c r="O5" s="5" t="n"/>
+      <c r="P5" s="5" t="n"/>
+      <c r="Q5" s="5" t="n"/>
+      <c r="R5" s="5" t="n"/>
+      <c r="S5" s="5" t="n"/>
+      <c r="T5" s="5" t="n"/>
+      <c r="U5" s="5" t="n"/>
+      <c r="V5" s="5" t="n"/>
+      <c r="W5" s="5" t="n"/>
+      <c r="X5" s="5" t="n"/>
+      <c r="Y5" s="5" t="n"/>
+      <c r="Z5" s="5" t="n"/>
+      <c r="AA5" s="5" t="n"/>
+      <c r="AB5" s="5" t="n"/>
+      <c r="AC5" s="5" t="n"/>
+      <c r="AD5" s="5" t="n"/>
+      <c r="AE5" s="5" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>boccella-rosa</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>boccella-rosa</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Boccella Rosa</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Boccella Rosa Azienda Vinicola</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>IT04567890123</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Giovanni Boccella</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>Il Taurasi è un vino che ha bisogno di tempo. Come le cose migliori.</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>castelfranci</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>Contrada Vigne 8, 83040 Castelfranci (AV)</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="n">
-        <v>40.93</v>
-      </c>
-      <c r="M6" s="5" t="n">
-        <v>15.04</v>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>PRODUTTORE_FOOD</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Vini d'Irpinia, anima di vulcano</t>
-        </is>
-      </c>
-      <c r="P6" s="5" t="inlineStr">
-        <is>
-          <t>Vini irpini d'eccellenza: Taurasi, Fiano e Greco di Tufo.</t>
-        </is>
-      </c>
-      <c r="Q6" s="5" t="inlineStr">
-        <is>
-          <t>Boccella Rosa nasce dalla passione di una famiglia di viticoltori che da generazioni coltiva i vitigni autoctoni dell'Irpinia. I vigneti di Aglianico, Fiano e Greco crescono su terreni vulcanici a 500 metri di altitudine, dove le escursioni termiche e i venti montani regalano uve di straordinaria intensità. La vinificazione rispetta i ritmi naturali, con lunghi affinamenti in botti di rovere e in bottiglia.</t>
-        </is>
-      </c>
-      <c r="R6" s="5" t="inlineStr">
-        <is>
-          <t>DOCG, DOC, BIO</t>
-        </is>
-      </c>
-      <c r="S6" s="5" t="inlineStr">
-        <is>
-          <t>2024 - Tre Bicchieri - Gambero Rosso | 2023 - 95 punti Taurasi Riserva - Wine Spectator</t>
-        </is>
-      </c>
-      <c r="T6" s="5" t="inlineStr">
-        <is>
-          <t>PLATINUM</t>
-        </is>
-      </c>
-      <c r="U6" s="5" t="inlineStr">
-        <is>
-          <t>info@boccellarosa.it</t>
-        </is>
-      </c>
-      <c r="V6" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 72145</t>
-        </is>
-      </c>
-      <c r="W6" s="5" t="inlineStr">
-        <is>
-          <t>https://boccellarosa.it</t>
-        </is>
-      </c>
-      <c r="X6" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y6" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Z6" s="5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/embed/dQw4w9WgXcQ</t>
-        </is>
-      </c>
-      <c r="AA6" s="5" t="inlineStr"/>
-      <c r="AB6" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC6" s="5" t="inlineStr">
-        <is>
-          <t>Export, Distribuzione, Enoteca, Ristorazione</t>
-        </is>
-      </c>
-      <c r="AD6" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE6" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="5" t="n"/>
+      <c r="O6" s="5" t="n"/>
+      <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="5" t="n"/>
+      <c r="R6" s="5" t="n"/>
+      <c r="S6" s="5" t="n"/>
+      <c r="T6" s="5" t="n"/>
+      <c r="U6" s="5" t="n"/>
+      <c r="V6" s="5" t="n"/>
+      <c r="W6" s="5" t="n"/>
+      <c r="X6" s="5" t="n"/>
+      <c r="Y6" s="5" t="n"/>
+      <c r="Z6" s="5" t="n"/>
+      <c r="AA6" s="5" t="n"/>
+      <c r="AB6" s="5" t="n"/>
+      <c r="AC6" s="5" t="n"/>
+      <c r="AD6" s="5" t="n"/>
+      <c r="AE6" s="5" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>re-del-bosco</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>re-del-bosco</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Re del Bosco</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Re del Bosco S.r.l.</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>IT05678901234</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>1990</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Luigi Montella</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Ogni castagna porta con sé il profumo del bosco e la pazienza dei nostri nonni.</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>montella</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>Via dei Castagneti 22, 83048 Montella (AV)</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="n">
-        <v>40.843</v>
-      </c>
-      <c r="M7" s="5" t="n">
-        <v>15.017</v>
-      </c>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>PRODUTTORE_FOOD</t>
-        </is>
-      </c>
-      <c r="O7" s="5" t="inlineStr">
-        <is>
-          <t>Le castagne più pregiate d'Italia</t>
-        </is>
-      </c>
-      <c r="P7" s="5" t="inlineStr">
-        <is>
-          <t>Castagna di Montella IGP e derivati dal cuore dei Picentini.</t>
-        </is>
-      </c>
-      <c r="Q7" s="5" t="inlineStr">
-        <is>
-          <t>Re del Bosco raccoglie e trasforma la Castagna di Montella IGP, una delle eccellenze più riconosciute della Campania. I castagneti secolari dei Monti Picentini, tra Montella e Bagnoli Irpino, producono frutti di dimensioni generose e sapore dolcissimo. Dall'essiccatura tradizionale nei "gratali" alla farina di castagne macinata a pietra, ogni prodotto preserva il gusto autentico del bosco irpino.</t>
-        </is>
-      </c>
-      <c r="R7" s="5" t="inlineStr">
-        <is>
-          <t>IGP, BIO</t>
-        </is>
-      </c>
-      <c r="S7" s="5" t="inlineStr">
-        <is>
-          <t>2024 - Premio Eccellenza IGP - Qualivita</t>
-        </is>
-      </c>
-      <c r="T7" s="5" t="inlineStr">
-        <is>
-          <t>PREMIUM</t>
-        </is>
-      </c>
-      <c r="U7" s="5" t="inlineStr">
-        <is>
-          <t>info@redelbosco.it</t>
-        </is>
-      </c>
-      <c r="V7" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 61234</t>
-        </is>
-      </c>
-      <c r="W7" s="5" t="inlineStr">
-        <is>
-          <t>https://www.redelbosco.it</t>
-        </is>
-      </c>
-      <c r="X7" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y7" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Z7" s="5" t="inlineStr"/>
-      <c r="AA7" s="5" t="inlineStr"/>
-      <c r="AB7" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC7" s="5" t="inlineStr">
-        <is>
-          <t>Distribuzione, Pasticceria, Export</t>
-        </is>
-      </c>
-      <c r="AD7" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE7" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="5" t="n"/>
+      <c r="O7" s="5" t="n"/>
+      <c r="P7" s="5" t="n"/>
+      <c r="Q7" s="5" t="n"/>
+      <c r="R7" s="5" t="n"/>
+      <c r="S7" s="5" t="n"/>
+      <c r="T7" s="5" t="n"/>
+      <c r="U7" s="5" t="n"/>
+      <c r="V7" s="5" t="n"/>
+      <c r="W7" s="5" t="n"/>
+      <c r="X7" s="5" t="n"/>
+      <c r="Y7" s="5" t="n"/>
+      <c r="Z7" s="5" t="n"/>
+      <c r="AA7" s="5" t="n"/>
+      <c r="AB7" s="5" t="n"/>
+      <c r="AC7" s="5" t="n"/>
+      <c r="AD7" s="5" t="n"/>
+      <c r="AE7" s="5" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>serrocroce</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>serrocroce</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Serrocroce</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Serrocroce Azienda Agricola</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>IT06789012345</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>2005</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Marco Serra</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Il vino naturale non si fa, si lascia fare. Noi ascoltiamo la vigna.</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>castelfranci</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>Contrada Serrocroce, 83040 Castelfranci (AV)</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="n">
-        <v>40.935</v>
-      </c>
-      <c r="M8" s="5" t="n">
-        <v>15.045</v>
-      </c>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>PRODUTTORE_FOOD</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>Vini naturali dall'Alta Irpinia</t>
-        </is>
-      </c>
-      <c r="P8" s="5" t="inlineStr">
-        <is>
-          <t>Vini naturali biodinamici da vigneti d'alta quota.</t>
-        </is>
-      </c>
-      <c r="Q8" s="5" t="inlineStr">
-        <is>
-          <t>Serrocroce è una cantina boutique che pratica viticoltura biodinamica sui terreni vulcanici dell'Alta Irpinia. I vigneti, coltivati a 600 metri sul livello del mare, producono vini di grande personalità: minerali, freschi, con una complessità aromatica che racconta il territorio. La cantina è scavata nel tufo, dove i vini riposano in anfore di terracotta e botti di castagno locale.</t>
-        </is>
-      </c>
-      <c r="R8" s="5" t="inlineStr">
-        <is>
-          <t>BIO, DOC</t>
-        </is>
-      </c>
-      <c r="S8" s="5" t="inlineStr">
-        <is>
-          <t>2024 - Vino Naturale dell'Anno - Guida Slow Wine</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr">
-        <is>
-          <t>BASE</t>
-        </is>
-      </c>
-      <c r="U8" s="5" t="inlineStr">
-        <is>
-          <t>info@serrocroce.it</t>
-        </is>
-      </c>
-      <c r="V8" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 72098</t>
-        </is>
-      </c>
-      <c r="W8" s="5" t="inlineStr">
-        <is>
-          <t>https://www.serrocroce.it</t>
-        </is>
-      </c>
-      <c r="X8" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y8" s="5" t="inlineStr"/>
-      <c r="Z8" s="5" t="inlineStr"/>
-      <c r="AA8" s="5" t="inlineStr"/>
-      <c r="AB8" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC8" s="5" t="inlineStr">
-        <is>
-          <t>Enoteca, Ristorazione, Export</t>
-        </is>
-      </c>
-      <c r="AD8" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE8" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
+      <c r="L8" s="5" t="n"/>
+      <c r="M8" s="5" t="n"/>
+      <c r="N8" s="5" t="n"/>
+      <c r="O8" s="5" t="n"/>
+      <c r="P8" s="5" t="n"/>
+      <c r="Q8" s="5" t="n"/>
+      <c r="R8" s="5" t="n"/>
+      <c r="S8" s="5" t="n"/>
+      <c r="T8" s="5" t="n"/>
+      <c r="U8" s="5" t="n"/>
+      <c r="V8" s="5" t="n"/>
+      <c r="W8" s="5" t="n"/>
+      <c r="X8" s="5" t="n"/>
+      <c r="Y8" s="5" t="n"/>
+      <c r="Z8" s="5" t="n"/>
+      <c r="AA8" s="5" t="n"/>
+      <c r="AB8" s="5" t="n"/>
+      <c r="AC8" s="5" t="n"/>
+      <c r="AD8" s="5" t="n"/>
+      <c r="AE8" s="5" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>caciocavalleria</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>caciocavalleria</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Caciocavalleria De D.</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Caciocavalleria De D. S.a.s.</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>IT07890123456</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>1975</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Paolo De Dominicis</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>Le nostre vacche Podoliche camminano libere. Il formaggio che producono non ha eguali.</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>lacedonia</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>Contrada Masseria 5, 83046 Lacedonia (AV)</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="n">
-        <v>41.05</v>
-      </c>
-      <c r="M9" s="5" t="n">
-        <v>15.42</v>
-      </c>
-      <c r="N9" s="5" t="inlineStr">
-        <is>
-          <t>PRODUTTORE_FOOD</t>
-        </is>
-      </c>
-      <c r="O9" s="5" t="inlineStr">
-        <is>
-          <t>Il re dei formaggi irpini</t>
-        </is>
-      </c>
-      <c r="P9" s="5" t="inlineStr">
-        <is>
-          <t>Caciocavallo Podolico e formaggi di latte crudo dall'Irpinia.</t>
-        </is>
-      </c>
-      <c r="Q9" s="5" t="inlineStr">
-        <is>
-          <t>La Caciocavalleria De D. è un caseificio artigianale specializzato nella produzione di Caciocavallo Podolico, ottenuto dal latte delle vacche Podoliche allevate al pascolo brado sui pascoli dell'Alta Irpinia. Questo formaggio raro, prodotto solo con latte di razza autoctona, viene stagionato per un minimo di 12 mesi nelle grotte naturali. Il risultato è un formaggio dal gusto intenso, leggermente piccante, con sentori di erbe selvatiche.</t>
-        </is>
-      </c>
-      <c r="R9" s="5" t="inlineStr">
-        <is>
-          <t>Slow Food, De.Co.</t>
-        </is>
-      </c>
-      <c r="S9" s="5" t="inlineStr">
-        <is>
-          <t>2023 - Presidio Slow Food - Slow Food Italia</t>
-        </is>
-      </c>
-      <c r="T9" s="5" t="inlineStr">
-        <is>
-          <t>PREMIUM</t>
-        </is>
-      </c>
-      <c r="U9" s="5" t="inlineStr">
-        <is>
-          <t>info@caciocavalleriaded.it</t>
-        </is>
-      </c>
-      <c r="V9" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 85012</t>
-        </is>
-      </c>
-      <c r="W9" s="5" t="inlineStr">
-        <is>
-          <t>https://www.caciocavalleriaded.it</t>
-        </is>
-      </c>
-      <c r="X9" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y9" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Z9" s="5" t="inlineStr"/>
-      <c r="AA9" s="5" t="inlineStr"/>
-      <c r="AB9" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC9" s="5" t="inlineStr">
-        <is>
-          <t>Distribuzione, Ristorazione, Export</t>
-        </is>
-      </c>
-      <c r="AD9" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE9" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
+      <c r="L9" s="5" t="n"/>
+      <c r="M9" s="5" t="n"/>
+      <c r="N9" s="5" t="n"/>
+      <c r="O9" s="5" t="n"/>
+      <c r="P9" s="5" t="n"/>
+      <c r="Q9" s="5" t="n"/>
+      <c r="R9" s="5" t="n"/>
+      <c r="S9" s="5" t="n"/>
+      <c r="T9" s="5" t="n"/>
+      <c r="U9" s="5" t="n"/>
+      <c r="V9" s="5" t="n"/>
+      <c r="W9" s="5" t="n"/>
+      <c r="X9" s="5" t="n"/>
+      <c r="Y9" s="5" t="n"/>
+      <c r="Z9" s="5" t="n"/>
+      <c r="AA9" s="5" t="n"/>
+      <c r="AB9" s="5" t="n"/>
+      <c r="AC9" s="5" t="n"/>
+      <c r="AD9" s="5" t="n"/>
+      <c r="AE9" s="5" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>carmasciando</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>carmasciando</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Carmasciando</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Carmasciando Azienda Agricola</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>IT08901234567</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>2010</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Salvatore Carmasciando</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Il vino è solo l'inizio. Venite a vivere questa terra.</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>torella-dei-lombardi</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>Contrada Piano 15, 83057 Torella dei Lombardi (AV)</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="n">
-        <v>40.94</v>
-      </c>
-      <c r="M10" s="5" t="n">
-        <v>15.113</v>
-      </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>MISTO</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr">
-        <is>
-          <t>Vino, terra, accoglienza</t>
-        </is>
-      </c>
-      <c r="P10" s="5" t="inlineStr">
-        <is>
-          <t>Cantina con agriturismo e esperienze nel cuore dell'Irpinia.</t>
-        </is>
-      </c>
-      <c r="Q10" s="5" t="inlineStr">
-        <is>
-          <t>Carmasciando è un progetto di vita che unisce viticoltura, ospitalità e cultura del territorio. La cantina produce vini da vitigni autoctoni irpini, mentre l'agriturismo offre esperienze immersive: dalle vendemmie partecipate alle cene in vigna, dalla raccolta delle olive ai laboratori di cucina irpina. Un luogo dove il tempo rallenta e i sapori raccontano storie.</t>
-        </is>
-      </c>
-      <c r="R10" s="5" t="inlineStr">
-        <is>
-          <t>BIO, DOC</t>
-        </is>
-      </c>
-      <c r="S10" s="5" t="inlineStr"/>
-      <c r="T10" s="5" t="inlineStr">
-        <is>
-          <t>PLATINUM</t>
-        </is>
-      </c>
-      <c r="U10" s="5" t="inlineStr">
-        <is>
-          <t>info@carmasciando.it</t>
-        </is>
-      </c>
-      <c r="V10" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 49876</t>
-        </is>
-      </c>
-      <c r="W10" s="5" t="inlineStr">
-        <is>
-          <t>https://carmasciando.it</t>
-        </is>
-      </c>
-      <c r="X10" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y10" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Z10" s="5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/embed/dQw4w9WgXcQ</t>
-        </is>
-      </c>
-      <c r="AA10" s="5" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/embed?pb=!4v1700000000000!6m8!1m7!1sCAoSLEFGMVFpcE5fX0JQX3RhbWVfY2FrRXdJOXJIeHFYVWNZb2JtVXdMbTBw!2m2!1d40.940!2d15.113!3f0!4f0!5f0.7820865974627469</t>
-        </is>
-      </c>
-      <c r="AB10" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC10" s="5" t="inlineStr">
-        <is>
-          <t>Turismo, Ristorazione, Eventi, Co-branding</t>
-        </is>
-      </c>
-      <c r="AD10" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE10" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
+      <c r="L10" s="5" t="n"/>
+      <c r="M10" s="5" t="n"/>
+      <c r="N10" s="5" t="n"/>
+      <c r="O10" s="5" t="n"/>
+      <c r="P10" s="5" t="n"/>
+      <c r="Q10" s="5" t="n"/>
+      <c r="R10" s="5" t="n"/>
+      <c r="S10" s="5" t="n"/>
+      <c r="T10" s="5" t="n"/>
+      <c r="U10" s="5" t="n"/>
+      <c r="V10" s="5" t="n"/>
+      <c r="W10" s="5" t="n"/>
+      <c r="X10" s="5" t="n"/>
+      <c r="Y10" s="5" t="n"/>
+      <c r="Z10" s="5" t="n"/>
+      <c r="AA10" s="5" t="n"/>
+      <c r="AB10" s="5" t="n"/>
+      <c r="AC10" s="5" t="n"/>
+      <c r="AD10" s="5" t="n"/>
+      <c r="AE10" s="5" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>torronificio-del-casale</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>torronificio-del-casale</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Torronificio del Casale</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Torronificio del Casale S.r.l.</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>IT09012345678</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>1890</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Rosa Del Casale</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Il segreto del nostro torrone? Il tempo. Non abbiamo mai avuto fretta.</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>sant-angelo-dei-lombardi</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>Via Mancini 8, 83054 Sant'Angelo dei Lombardi (AV)</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="n">
-        <v>40.927</v>
-      </c>
-      <c r="M11" s="5" t="n">
-        <v>15.175</v>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>PRODUTTORE_FOOD</t>
-        </is>
-      </c>
-      <c r="O11" s="5" t="inlineStr">
-        <is>
-          <t>L'arte del torrone dal 1890</t>
-        </is>
-      </c>
-      <c r="P11" s="5" t="inlineStr">
-        <is>
-          <t>Torroni artigianali irpini: miele, nocciole e tradizione.</t>
-        </is>
-      </c>
-      <c r="Q11" s="5" t="inlineStr">
-        <is>
-          <t>Il Torronificio del Casale porta avanti una tradizione dolciaria che risale alla fine dell'Ottocento. Il torrone viene prodotto con miele di castagno dell'Irpinia, nocciole Tonde di Giffoni e mandorle selezionate, seguendo il metodo di cottura lenta in caldaie di rame. Ogni barretta è confezionata a mano, come si faceva un tempo. Una dolcezza autentica che racconta la storia del Natale irpino.</t>
-        </is>
-      </c>
-      <c r="R11" s="5" t="inlineStr">
-        <is>
-          <t>De.Co., Slow Food</t>
-        </is>
-      </c>
-      <c r="S11" s="5" t="inlineStr">
-        <is>
-          <t>2024 - Eccellenza Artigiana - CNA Campania</t>
-        </is>
-      </c>
-      <c r="T11" s="5" t="inlineStr">
-        <is>
-          <t>PREMIUM</t>
-        </is>
-      </c>
-      <c r="U11" s="5" t="inlineStr">
-        <is>
-          <t>info@torronificiodelcasale.com</t>
-        </is>
-      </c>
-      <c r="V11" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 23456</t>
-        </is>
-      </c>
-      <c r="W11" s="5" t="inlineStr">
-        <is>
-          <t>https://www.torronificiodelcasale.com</t>
-        </is>
-      </c>
-      <c r="X11" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y11" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Z11" s="5" t="inlineStr"/>
-      <c r="AA11" s="5" t="inlineStr"/>
-      <c r="AB11" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC11" s="5" t="inlineStr">
-        <is>
-          <t>Distribuzione, Gift box, Export, HoReCa</t>
-        </is>
-      </c>
-      <c r="AD11" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE11" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
+      <c r="L11" s="5" t="n"/>
+      <c r="M11" s="5" t="n"/>
+      <c r="N11" s="5" t="n"/>
+      <c r="O11" s="5" t="n"/>
+      <c r="P11" s="5" t="n"/>
+      <c r="Q11" s="5" t="n"/>
+      <c r="R11" s="5" t="n"/>
+      <c r="S11" s="5" t="n"/>
+      <c r="T11" s="5" t="n"/>
+      <c r="U11" s="5" t="n"/>
+      <c r="V11" s="5" t="n"/>
+      <c r="W11" s="5" t="n"/>
+      <c r="X11" s="5" t="n"/>
+      <c r="Y11" s="5" t="n"/>
+      <c r="Z11" s="5" t="n"/>
+      <c r="AA11" s="5" t="n"/>
+      <c r="AB11" s="5" t="n"/>
+      <c r="AC11" s="5" t="n"/>
+      <c r="AD11" s="5" t="n"/>
+      <c r="AE11" s="5" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>dolci-terre</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>dolci-terre</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Dolci Terre</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Dolci Terre di Irpinia</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>IT10123456789</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>2008</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>Francesca Iannaccone</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>La natura ci regala tutto. Noi lo mettiamo in un vasetto.</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>montella</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>Via Fontana 30, 83048 Montella (AV)</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="n">
-        <v>40.845</v>
-      </c>
-      <c r="M12" s="5" t="n">
-        <v>15.02</v>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>PRODUTTORE_FOOD</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>La dolcezza autentica dell'Irpinia</t>
-        </is>
-      </c>
-      <c r="P12" s="5" t="inlineStr">
-        <is>
-          <t>Confetture, mieli e conserve dal cuore verde dell'Irpinia.</t>
-        </is>
-      </c>
-      <c r="Q12" s="5" t="inlineStr">
-        <is>
-          <t>Dolci Terre trasforma i frutti spontanei e coltivati dell'Alta Irpinia in confetture, mieli aromatici e conserve. Dalle fichi tardive ai pomodori secchi, dal miele di castagno a quello millefiori di montagna: ogni vasetto è il risultato di una filiera cortissima, dalla pianta al prodotto finito in meno di 48 ore. Senza conservanti, senza coloranti, solo il sapore vero della terra.</t>
-        </is>
-      </c>
-      <c r="R12" s="5" t="inlineStr">
-        <is>
-          <t>BIO</t>
-        </is>
-      </c>
-      <c r="S12" s="5" t="inlineStr"/>
-      <c r="T12" s="5" t="inlineStr">
-        <is>
-          <t>BASE</t>
-        </is>
-      </c>
-      <c r="U12" s="5" t="inlineStr">
-        <is>
-          <t>info@dolciterre.it</t>
-        </is>
-      </c>
-      <c r="V12" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 61890</t>
-        </is>
-      </c>
-      <c r="W12" s="5" t="inlineStr">
-        <is>
-          <t>https://www.dolciterre.it</t>
-        </is>
-      </c>
-      <c r="X12" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y12" s="5" t="inlineStr"/>
-      <c r="Z12" s="5" t="inlineStr"/>
-      <c r="AA12" s="5" t="inlineStr"/>
-      <c r="AB12" s="5" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="AC12" s="5" t="inlineStr"/>
-      <c r="AD12" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE12" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="5" t="n"/>
+      <c r="L12" s="5" t="n"/>
+      <c r="M12" s="5" t="n"/>
+      <c r="N12" s="5" t="n"/>
+      <c r="O12" s="5" t="n"/>
+      <c r="P12" s="5" t="n"/>
+      <c r="Q12" s="5" t="n"/>
+      <c r="R12" s="5" t="n"/>
+      <c r="S12" s="5" t="n"/>
+      <c r="T12" s="5" t="n"/>
+      <c r="U12" s="5" t="n"/>
+      <c r="V12" s="5" t="n"/>
+      <c r="W12" s="5" t="n"/>
+      <c r="X12" s="5" t="n"/>
+      <c r="Y12" s="5" t="n"/>
+      <c r="Z12" s="5" t="n"/>
+      <c r="AA12" s="5" t="n"/>
+      <c r="AB12" s="5" t="n"/>
+      <c r="AC12" s="5" t="n"/>
+      <c r="AD12" s="5" t="n"/>
+      <c r="AE12" s="5" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>tenuta-pepe</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>tenuta-pepe</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Tenuta Pepe</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Tenuta Pepe S.a.s.</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>IT11234567890</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>1986</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Roberto Pepe</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>L'Irpinia è la Borgogna del Sud. I nostri vini lo dimostrano.</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>lioni</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>Contrada Vigne 5, 83047 Lioni (AV)</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="n">
-        <v>40.878</v>
-      </c>
-      <c r="M13" s="5" t="n">
-        <v>15.183</v>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>PRODUTTORE_FOOD</t>
-        </is>
-      </c>
-      <c r="O13" s="5" t="inlineStr">
-        <is>
-          <t>Tradizione vinicola dal 1986</t>
-        </is>
-      </c>
-      <c r="P13" s="5" t="inlineStr">
-        <is>
-          <t>Vini d'autore dall'Irpinia: Taurasi DOCG e Fiano di Avellino.</t>
-        </is>
-      </c>
-      <c r="Q13" s="5" t="inlineStr">
-        <is>
-          <t>Tenuta Pepe è una delle cantine storiche dell'Irpinia, fondata nel 1986 dalla famiglia Pepe con l'obiettivo di valorizzare i grandi vitigni autoctoni campani. I vigneti si estendono su 15 ettari di terreni argilloso-calcarei, ideali per l'Aglianico e il Fiano. La cantina combina metodi tradizionali con tecnologia enologica moderna, producendo vini eleganti che esprimono il terroir irpino.</t>
-        </is>
-      </c>
-      <c r="R13" s="5" t="inlineStr">
-        <is>
-          <t>DOCG, DOC, BIO</t>
-        </is>
-      </c>
-      <c r="S13" s="5" t="inlineStr">
-        <is>
-          <t>2024 - Tre Bicchieri Taurasi - Gambero Rosso | 2023 - 93 punti Fiano - James Suckling</t>
-        </is>
-      </c>
-      <c r="T13" s="5" t="inlineStr">
-        <is>
-          <t>PLATINUM</t>
-        </is>
-      </c>
-      <c r="U13" s="5" t="inlineStr">
-        <is>
-          <t>info@tenutapepe.it</t>
-        </is>
-      </c>
-      <c r="V13" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 42567</t>
-        </is>
-      </c>
-      <c r="W13" s="5" t="inlineStr">
-        <is>
-          <t>https://www.tenutapepe.it</t>
-        </is>
-      </c>
-      <c r="X13" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y13" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Z13" s="5" t="inlineStr"/>
-      <c r="AA13" s="5" t="inlineStr"/>
-      <c r="AB13" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC13" s="5" t="inlineStr">
-        <is>
-          <t>Export, Enoteca, Ristorazione, Hotel</t>
-        </is>
-      </c>
-      <c r="AD13" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE13" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
+      <c r="M13" s="5" t="n"/>
+      <c r="N13" s="5" t="n"/>
+      <c r="O13" s="5" t="n"/>
+      <c r="P13" s="5" t="n"/>
+      <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="5" t="n"/>
+      <c r="S13" s="5" t="n"/>
+      <c r="T13" s="5" t="n"/>
+      <c r="U13" s="5" t="n"/>
+      <c r="V13" s="5" t="n"/>
+      <c r="W13" s="5" t="n"/>
+      <c r="X13" s="5" t="n"/>
+      <c r="Y13" s="5" t="n"/>
+      <c r="Z13" s="5" t="n"/>
+      <c r="AA13" s="5" t="n"/>
+      <c r="AB13" s="5" t="n"/>
+      <c r="AC13" s="5" t="n"/>
+      <c r="AD13" s="5" t="n"/>
+      <c r="AE13" s="5" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>sella-delle-spine</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>sella-delle-spine</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Sella delle Spine</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Sella delle Spine Azienda Agricola</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>IT12345678901</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>1998</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>Anna Spinelli</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>Il Greco di Tufo è la voce della terra vulcanica. Noi lo lasciamo parlare.</t>
-        </is>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>calitri</t>
-        </is>
-      </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>Contrada Spine 3, 83045 Calitri (AV)</t>
-        </is>
-      </c>
-      <c r="L14" s="5" t="n">
-        <v>40.9</v>
-      </c>
-      <c r="M14" s="5" t="n">
-        <v>15.44</v>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>PRODUTTORE_FOOD</t>
-        </is>
-      </c>
-      <c r="O14" s="5" t="inlineStr">
-        <is>
-          <t>Dove nasce il Greco di Tufo</t>
-        </is>
-      </c>
-      <c r="P14" s="5" t="inlineStr">
-        <is>
-          <t>Greco di Tufo DOCG e bianchi d'alta quota.</t>
-        </is>
-      </c>
-      <c r="Q14" s="5" t="inlineStr">
-        <is>
-          <t>Sella delle Spine è una piccola cantina familiare che coltiva Greco di Tufo sui pendii vulcanici dell'Irpinia. I vigneti, esposti a sud-est, beneficiano delle brezze montane e delle escursioni termiche che conferiscono al Greco una freschezza e una mineralità uniche. La produzione è volutamente limitata per garantire la massima qualità in ogni bottiglia.</t>
-        </is>
-      </c>
-      <c r="R14" s="5" t="inlineStr">
-        <is>
-          <t>DOCG, BIO</t>
-        </is>
-      </c>
-      <c r="S14" s="5" t="inlineStr"/>
-      <c r="T14" s="5" t="inlineStr">
-        <is>
-          <t>BASE</t>
-        </is>
-      </c>
-      <c r="U14" s="5" t="inlineStr">
-        <is>
-          <t>info@selladellespine.com</t>
-        </is>
-      </c>
-      <c r="V14" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 35012</t>
-        </is>
-      </c>
-      <c r="W14" s="5" t="inlineStr">
-        <is>
-          <t>https://www.selladellespine.com</t>
-        </is>
-      </c>
-      <c r="X14" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y14" s="5" t="inlineStr"/>
-      <c r="Z14" s="5" t="inlineStr"/>
-      <c r="AA14" s="5" t="inlineStr"/>
-      <c r="AB14" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC14" s="5" t="inlineStr">
-        <is>
-          <t>Enoteca, Export</t>
-        </is>
-      </c>
-      <c r="AD14" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE14" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="5" t="n"/>
+      <c r="L14" s="5" t="n"/>
+      <c r="M14" s="5" t="n"/>
+      <c r="N14" s="5" t="n"/>
+      <c r="O14" s="5" t="n"/>
+      <c r="P14" s="5" t="n"/>
+      <c r="Q14" s="5" t="n"/>
+      <c r="R14" s="5" t="n"/>
+      <c r="S14" s="5" t="n"/>
+      <c r="T14" s="5" t="n"/>
+      <c r="U14" s="5" t="n"/>
+      <c r="V14" s="5" t="n"/>
+      <c r="W14" s="5" t="n"/>
+      <c r="X14" s="5" t="n"/>
+      <c r="Y14" s="5" t="n"/>
+      <c r="Z14" s="5" t="n"/>
+      <c r="AA14" s="5" t="n"/>
+      <c r="AB14" s="5" t="n"/>
+      <c r="AC14" s="5" t="n"/>
+      <c r="AD14" s="5" t="n"/>
+      <c r="AE14" s="5" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>bifulco</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>bifulco</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Bifulco</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Bifulco Alimentari S.r.l.</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>IT13456789012</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>1972</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Carlo Bifulco</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>La pasta buona si riconosce dal profumo del grano, non dall'etichetta.</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>lioni</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>Via Industria 18, 83047 Lioni (AV)</t>
-        </is>
-      </c>
-      <c r="L15" s="5" t="n">
-        <v>40.88</v>
-      </c>
-      <c r="M15" s="5" t="n">
-        <v>15.185</v>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>PRODUTTORE_FOOD</t>
-        </is>
-      </c>
-      <c r="O15" s="5" t="inlineStr">
-        <is>
-          <t>Pasta e tradizione irpina</t>
-        </is>
-      </c>
-      <c r="P15" s="5" t="inlineStr">
-        <is>
-          <t>Pasta artigianale e prodotti da forno della tradizione irpina.</t>
-        </is>
-      </c>
-      <c r="Q15" s="5" t="inlineStr">
-        <is>
-          <t>Bifulco è un pastificio artigianale che produce pasta di semola di grano duro con trafilatura al bronzo e essiccazione lenta. I fusilli al ferretto, i cavatelli e le lagane sono le specialità della casa, preparate con lo stesso metodo che le massaie irpine usano da secoli. Il grano proviene dalle campagne dell'Alta Irpinia, macinato in piccoli mulini locali.</t>
-        </is>
-      </c>
-      <c r="R15" s="5" t="inlineStr">
-        <is>
-          <t>De.Co.</t>
-        </is>
-      </c>
-      <c r="S15" s="5" t="inlineStr"/>
-      <c r="T15" s="5" t="inlineStr">
-        <is>
-          <t>BASE</t>
-        </is>
-      </c>
-      <c r="U15" s="5" t="inlineStr">
-        <is>
-          <t>info@bifulco.it</t>
-        </is>
-      </c>
-      <c r="V15" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 42890</t>
-        </is>
-      </c>
-      <c r="W15" s="5" t="inlineStr">
-        <is>
-          <t>https://www.bifulco.it</t>
-        </is>
-      </c>
-      <c r="X15" s="5" t="inlineStr"/>
-      <c r="Y15" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Z15" s="5" t="inlineStr"/>
-      <c r="AA15" s="5" t="inlineStr"/>
-      <c r="AB15" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC15" s="5" t="inlineStr">
-        <is>
-          <t>Distribuzione, Ristorazione</t>
-        </is>
-      </c>
-      <c r="AD15" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE15" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
+      <c r="L15" s="5" t="n"/>
+      <c r="M15" s="5" t="n"/>
+      <c r="N15" s="5" t="n"/>
+      <c r="O15" s="5" t="n"/>
+      <c r="P15" s="5" t="n"/>
+      <c r="Q15" s="5" t="n"/>
+      <c r="R15" s="5" t="n"/>
+      <c r="S15" s="5" t="n"/>
+      <c r="T15" s="5" t="n"/>
+      <c r="U15" s="5" t="n"/>
+      <c r="V15" s="5" t="n"/>
+      <c r="W15" s="5" t="n"/>
+      <c r="X15" s="5" t="n"/>
+      <c r="Y15" s="5" t="n"/>
+      <c r="Z15" s="5" t="n"/>
+      <c r="AA15" s="5" t="n"/>
+      <c r="AB15" s="5" t="n"/>
+      <c r="AC15" s="5" t="n"/>
+      <c r="AD15" s="5" t="n"/>
+      <c r="AE15" s="5" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>akudunniad</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>akudunniad</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>A' Ku Dunniad</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>A' Ku Dunniad Cooperativa Sociale</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>IT14567890123</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>2015</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Teresa Calitri</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>Restare è la forma più coraggiosa di innovazione.</t>
-        </is>
-      </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>calitri</t>
-        </is>
-      </c>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>Via del Borgo 7, 83045 Calitri (AV)</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="n">
-        <v>40.895</v>
-      </c>
-      <c r="M16" s="5" t="n">
-        <v>15.435</v>
-      </c>
-      <c r="N16" s="5" t="inlineStr">
-        <is>
-          <t>MISTO</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr">
-        <is>
-          <t>Il sapore della comunità</t>
-        </is>
-      </c>
-      <c r="P16" s="5" t="inlineStr">
-        <is>
-          <t>Cooperativa sociale: prodotti tipici, ospitalità e inclusione.</t>
-        </is>
-      </c>
-      <c r="Q16" s="5" t="inlineStr">
-        <is>
-          <t>A' Ku Dunniad (dal dialetto irpino "come una volta") è una cooperativa sociale che unisce produzione agroalimentare, turismo responsabile e inclusione sociale. I prodotti — conserve, confetture, pasta fresca — nascono dal lavoro di una comunità che ha scelto di restare e innovare nei borghi dell'Alta Irpinia. Un modello di economia circolare e sostenibile.</t>
-        </is>
-      </c>
-      <c r="R16" s="5" t="inlineStr">
-        <is>
-          <t>BIO</t>
-        </is>
-      </c>
-      <c r="S16" s="5" t="inlineStr">
-        <is>
-          <t>2023 - Premio Innovazione Sociale - Ashoka Italia</t>
-        </is>
-      </c>
-      <c r="T16" s="5" t="inlineStr">
-        <is>
-          <t>PREMIUM</t>
-        </is>
-      </c>
-      <c r="U16" s="5" t="inlineStr">
-        <is>
-          <t>info@akudunniad.it</t>
-        </is>
-      </c>
-      <c r="V16" s="5" t="inlineStr">
-        <is>
-          <t>+39 0827 35890</t>
-        </is>
-      </c>
-      <c r="W16" s="5" t="inlineStr">
-        <is>
-          <t>https://akudunniad.it</t>
-        </is>
-      </c>
-      <c r="X16" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Y16" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="Z16" s="5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/embed/dQw4w9WgXcQ</t>
-        </is>
-      </c>
-      <c r="AA16" s="5" t="inlineStr"/>
-      <c r="AB16" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AC16" s="5" t="inlineStr">
-        <is>
-          <t>Turismo, Inclusione sociale, Distribuzione</t>
-        </is>
-      </c>
-      <c r="AD16" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AE16" s="5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="A16" s="5" t="n"/>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
+      <c r="L16" s="5" t="n"/>
+      <c r="M16" s="5" t="n"/>
+      <c r="N16" s="5" t="n"/>
+      <c r="O16" s="5" t="n"/>
+      <c r="P16" s="5" t="n"/>
+      <c r="Q16" s="5" t="n"/>
+      <c r="R16" s="5" t="n"/>
+      <c r="S16" s="5" t="n"/>
+      <c r="T16" s="5" t="n"/>
+      <c r="U16" s="5" t="n"/>
+      <c r="V16" s="5" t="n"/>
+      <c r="W16" s="5" t="n"/>
+      <c r="X16" s="5" t="n"/>
+      <c r="Y16" s="5" t="n"/>
+      <c r="Z16" s="5" t="n"/>
+      <c r="AA16" s="5" t="n"/>
+      <c r="AB16" s="5" t="n"/>
+      <c r="AC16" s="5" t="n"/>
+      <c r="AD16" s="5" t="n"/>
+      <c r="AE16" s="5" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="5" t="n"/>
@@ -4624,45 +3405,177 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
-      <c r="P4" s="5" t="n"/>
-      <c r="Q4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
-      <c r="S4" s="5" t="n"/>
-      <c r="T4" s="5" t="n"/>
-      <c r="U4" s="5" t="n"/>
-      <c r="V4" s="5" t="n"/>
-      <c r="W4" s="5" t="n"/>
-      <c r="X4" s="5" t="n"/>
-      <c r="Y4" s="5" t="n"/>
-      <c r="Z4" s="5" t="n"/>
-      <c r="AA4" s="5" t="n"/>
-      <c r="AB4" s="5" t="n"/>
-      <c r="AC4" s="5" t="n"/>
-      <c r="AD4" s="5" t="n"/>
-      <c r="AE4" s="5" t="n"/>
-      <c r="AF4" s="5" t="n"/>
-      <c r="AG4" s="5" t="n"/>
-      <c r="AH4" s="5" t="n"/>
-      <c r="AI4" s="5" t="n"/>
-      <c r="AJ4" s="5" t="n"/>
-      <c r="AK4" s="5" t="n"/>
-      <c r="AL4" s="5" t="n"/>
-      <c r="AM4" s="5" t="n"/>
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>tour-caseificio</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>tour-caseificio-caciocavallo-podolico</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Il Caciocavallo Podolico: Dal Pascolo alla Tavola</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Un formaggio raro, una storia millenaria</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>GASTRONOMIA</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>caciocavalleria</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>lacedonia</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Visita al caseificio artigianale con mungitura, caseificazione dal vivo e degustazione guidata di 5 stagionature.</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>Scopri il segreto del Caciocavallo Podolico, uno dei formaggi più rari d'Italia, nella Caciocavalleria De D. a Lacedonia. La giornata inizia con la visita ai pascoli dove le vacche Podoliche brucano libere. Si prosegue con la dimostrazione di caseificazione dal vivo. La visita si conclude nelle grotte di stagionatura in tufo. Degustazione finale di 5 stagionature diverse (3, 6, 12, 18 e 24 mesi), accompagnate da miele di castagno e confettura di fichi.</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="n">
+        <v>180</v>
+      </c>
+      <c r="K4" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="L4" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" s="15" t="n">
+        <v>55</v>
+      </c>
+      <c r="N4" s="15" t="inlineStr">
+        <is>
+          <t>FACILE</t>
+        </is>
+      </c>
+      <c r="O4" s="15" t="inlineStr">
+        <is>
+          <t>Italiano</t>
+        </is>
+      </c>
+      <c r="P4" s="15" t="inlineStr">
+        <is>
+          <t>Visita pascoli|Dimostrazione caseificazione|Degustazione 5 stagionature|Miele e confettura|Forma di caciocavallo giovane omaggio</t>
+        </is>
+      </c>
+      <c r="Q4" s="15" t="inlineStr">
+        <is>
+          <t>Trasporto|Pranzo</t>
+        </is>
+      </c>
+      <c r="R4" s="15" t="inlineStr">
+        <is>
+          <t>Scarpe da campagna|Abbigliamento comodo</t>
+        </is>
+      </c>
+      <c r="S4" s="15" t="inlineStr">
+        <is>
+          <t>Cancellazione gratuita fino a 48 ore prima.</t>
+        </is>
+      </c>
+      <c r="T4" s="15" t="inlineStr">
+        <is>
+          <t>Cantina accessibile con rampa. Visita pascoli su terreno non pavimentato.</t>
+        </is>
+      </c>
+      <c r="U4" s="15" t="inlineStr">
+        <is>
+          <t>primavera, estate, autunno</t>
+        </is>
+      </c>
+      <c r="V4" s="15" t="n">
+        <v>41.05</v>
+      </c>
+      <c r="W4" s="15" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="X4" s="15" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="Y4" s="15" t="inlineStr">
+        <is>
+          <t>Pascoli</t>
+        </is>
+      </c>
+      <c r="Z4" s="15" t="inlineStr">
+        <is>
+          <t>Visita alle vacche Podoliche al pascolo</t>
+        </is>
+      </c>
+      <c r="AA4" s="15" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="AB4" s="15" t="inlineStr">
+        <is>
+          <t>Caseificazione</t>
+        </is>
+      </c>
+      <c r="AC4" s="15" t="inlineStr">
+        <is>
+          <t>Dimostrazione di cagliatura e filatura a mano</t>
+        </is>
+      </c>
+      <c r="AD4" s="15" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="AE4" s="15" t="inlineStr">
+        <is>
+          <t>Grotte di stagionatura</t>
+        </is>
+      </c>
+      <c r="AF4" s="15" t="inlineStr">
+        <is>
+          <t>Visita alle grotte in tufo con formaggi in affinamento</t>
+        </is>
+      </c>
+      <c r="AG4" s="15" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="AH4" s="15" t="inlineStr">
+        <is>
+          <t>Degustazione</t>
+        </is>
+      </c>
+      <c r="AI4" s="15" t="inlineStr">
+        <is>
+          <t>5 stagionature con miele e confettura</t>
+        </is>
+      </c>
+      <c r="AJ4" s="15" t="inlineStr"/>
+      <c r="AK4" s="15" t="inlineStr"/>
+      <c r="AL4" s="15" t="inlineStr"/>
+      <c r="AM4" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="n"/>
@@ -7112,36 +6025,124 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
-      <c r="P4" s="5" t="n"/>
-      <c r="Q4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
-      <c r="S4" s="5" t="n"/>
-      <c r="T4" s="5" t="n"/>
-      <c r="U4" s="5" t="n"/>
-      <c r="V4" s="5" t="n"/>
-      <c r="W4" s="5" t="n"/>
-      <c r="X4" s="5" t="n"/>
-      <c r="Y4" s="5" t="n"/>
-      <c r="Z4" s="5" t="n"/>
-      <c r="AA4" s="5" t="n"/>
-      <c r="AB4" s="5" t="n"/>
-      <c r="AC4" s="5" t="n"/>
-      <c r="AD4" s="5" t="n"/>
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>cesto-vimini-lacedonia</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>cesto-vimini-tradizionale-lacedonia</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Cesto in Vimini per Raccolta Tradizionale</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>akudunniad</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>lacedonia</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Cesto intrecciato a mano in vimini locale, perfetto per raccolta e decorazione.</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Cesto tradizionale intrecciato a mano con vimini raccolto lungo i fiumi dell'Irpinia. La tecnica di intreccio è quella tramandata dai contadini per la raccolta di castagne, olive e uva. Il manico rinforzato permette di trasportare carichi pesanti. Ogni cesto è unico per le variazioni naturali del vimini.</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Intreccio a mano con tecnica tradizionale, manico rinforzato</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>vimini</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="n">
+        <v>42</v>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>diam. 35 cm x h 25 cm (con manico h 40 cm)</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="n">
+        <v>450</v>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="N4" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="O4" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="P4" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q4" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="R4" s="15" t="inlineStr">
+        <is>
+          <t>Dimensione</t>
+        </is>
+      </c>
+      <c r="S4" s="15" t="inlineStr">
+        <is>
+          <t>Piccolo diam.25, Medio diam.35, Grande diam.45</t>
+        </is>
+      </c>
+      <c r="T4" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="U4" s="15" t="inlineStr"/>
+      <c r="V4" s="15" t="inlineStr"/>
+      <c r="W4" s="15" t="inlineStr"/>
+      <c r="X4" s="15" t="inlineStr">
+        <is>
+          <t>Raccolta vimini</t>
+        </is>
+      </c>
+      <c r="Y4" s="15" t="inlineStr">
+        <is>
+          <t>Vimini locale raccolto in inverno lungo i fiumi</t>
+        </is>
+      </c>
+      <c r="Z4" s="15" t="inlineStr">
+        <is>
+          <t>Intreccio</t>
+        </is>
+      </c>
+      <c r="AA4" s="15" t="inlineStr">
+        <is>
+          <t>Intreccio a mano con tecnica tradizionale</t>
+        </is>
+      </c>
+      <c r="AB4" s="15" t="inlineStr"/>
+      <c r="AC4" s="15" t="inlineStr"/>
+      <c r="AD4" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="n"/>
@@ -9074,30 +8075,116 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
-      <c r="P4" s="5" t="n"/>
-      <c r="Q4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
-      <c r="S4" s="5" t="n"/>
-      <c r="T4" s="5" t="n"/>
-      <c r="U4" s="5" t="n"/>
-      <c r="V4" s="5" t="n"/>
-      <c r="W4" s="5" t="n"/>
-      <c r="X4" s="5" t="n"/>
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>caciocavallo-podolico-18m</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>caciocavallo-podolico-18m</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Caciocavallo Podolico 18 Mesi</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>caciocavalleria</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>lacedonia</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>FORMAGGI</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Il re dei formaggi irpini: Caciocavallo Podolico stagionato 18 mesi in grotta di tufo.</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Il Caciocavallo Podolico della Caciocavalleria De D. è un formaggio raro e prezioso, prodotto esclusivamente con latte crudo di vacche Podoliche allevate al pascolo brado sui pascoli dell'Alta Irpinia. La cagliatura tradizionale e la stagionatura di 18 mesi nelle grotte naturali in tufo conferiscono un sapore intenso e complesso: note di erbe selvatiche, nocciola, burro fuso e un leggero piccante che si attenua nel finale lungo e persistente.</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>Il re dei formaggi del Sud</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>Miele di castagno, confettura di fichi, Taurasi DOCG</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>pezzo (ca. 1.2 kg)</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="n">
+        <v>1200</v>
+      </c>
+      <c r="N4" s="15" t="n">
+        <v>180</v>
+      </c>
+      <c r="O4" s="15" t="inlineStr">
+        <is>
+          <t>Conservare in luogo fresco e asciutto, avvolto in carta alimentare</t>
+        </is>
+      </c>
+      <c r="P4" s="15" t="inlineStr">
+        <is>
+          <t>Presidio Slow Food</t>
+        </is>
+      </c>
+      <c r="Q4" s="15" t="inlineStr">
+        <is>
+          <t>Latte</t>
+        </is>
+      </c>
+      <c r="R4" s="15" t="inlineStr">
+        <is>
+          <t>Latte crudo di vacca Podolica, caglio naturale, sale</t>
+        </is>
+      </c>
+      <c r="S4" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="T4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="U4" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="V4" s="15" t="inlineStr">
+        <is>
+          <t>Spedizione in confezione isotermica</t>
+        </is>
+      </c>
+      <c r="W4" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="X4" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="n"/>
@@ -10838,37 +9925,135 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
-      <c r="P4" s="5" t="n"/>
-      <c r="Q4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
-      <c r="S4" s="5" t="n"/>
-      <c r="T4" s="5" t="n"/>
-      <c r="U4" s="5" t="n"/>
-      <c r="V4" s="5" t="n"/>
-      <c r="W4" s="5" t="n"/>
-      <c r="X4" s="5" t="n"/>
-      <c r="Y4" s="5" t="n"/>
-      <c r="Z4" s="5" t="n"/>
-      <c r="AA4" s="5" t="n"/>
-      <c r="AB4" s="5" t="n"/>
-      <c r="AC4" s="5" t="n"/>
-      <c r="AD4" s="5" t="n"/>
-      <c r="AE4" s="5" t="n"/>
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>masseria-lacedonia</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>masseria-santa-lucia-lacedonia</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Masseria Santa Lucia</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>MASSERIA</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>caciocavalleria</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>lacedonia</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Contrada Masseria 5, 83046 Lacedonia (AV)</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="n">
+        <v>41.05</v>
+      </c>
+      <c r="I4" s="15" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="J4" s="15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>Masseria storica immersa nei pascoli dell'Alta Irpinia, a due passi dal caseificio del Caciocavallo Podolico.</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>Masseria Santa Lucia è un'antica masseria ristrutturata che offre un'esperienza di soggiorno autentica nel cuore dell'Alta Irpinia. Le camere, ricavate dalle antiche stalle e dai fienili, conservano le volte in pietra e i pavimenti in cotto originali. La colazione è a base di prodotti del caseificio e dell'orto aziendale. Posizione ideale per esplorare Lacedonia e i borghi circostanti.</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>Dormire tra storia e pascoli</t>
+        </is>
+      </c>
+      <c r="N4" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="O4" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="P4" s="15" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q4" s="15" t="inlineStr">
+        <is>
+          <t>Agriturismo 3 spighe</t>
+        </is>
+      </c>
+      <c r="R4" s="15" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="S4" s="15" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="T4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="U4" s="15" t="inlineStr">
+        <is>
+          <t>WiFi, Parcheggio, Colazione inclusa, Giardino, Animali ammessi</t>
+        </is>
+      </c>
+      <c r="V4" s="15" t="inlineStr">
+        <is>
+          <t>Piano terra accessibile</t>
+        </is>
+      </c>
+      <c r="W4" s="15" t="inlineStr">
+        <is>
+          <t>Italiano, English</t>
+        </is>
+      </c>
+      <c r="X4" s="15" t="inlineStr">
+        <is>
+          <t>Cancellazione gratuita fino a 48 ore prima</t>
+        </is>
+      </c>
+      <c r="Y4" s="15" t="inlineStr">
+        <is>
+          <t>booking@caciocavalleriaded.it</t>
+        </is>
+      </c>
+      <c r="Z4" s="15" t="inlineStr">
+        <is>
+          <t>+39 0827 85012</t>
+        </is>
+      </c>
+      <c r="AA4" s="15" t="inlineStr"/>
+      <c r="AB4" s="15" t="inlineStr"/>
+      <c r="AC4" s="15" t="inlineStr"/>
+      <c r="AD4" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE4" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="n"/>
@@ -12508,6 +11693,594 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AE4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="31" max="31"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>🍽️ ANAGRAFICA</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="n"/>
+      <c r="C1" s="17" t="n"/>
+      <c r="D1" s="17" t="n"/>
+      <c r="E1" s="16" t="inlineStr">
+        <is>
+          <t>📍 LOCALIZZAZIONE</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="n"/>
+      <c r="G1" s="17" t="n"/>
+      <c r="H1" s="17" t="n"/>
+      <c r="I1" s="16" t="inlineStr">
+        <is>
+          <t>📝 DESCRIZIONI</t>
+        </is>
+      </c>
+      <c r="J1" s="17" t="n"/>
+      <c r="K1" s="17" t="n"/>
+      <c r="L1" s="16" t="inlineStr">
+        <is>
+          <t>⚙️ DETTAGLI</t>
+        </is>
+      </c>
+      <c r="M1" s="17" t="n"/>
+      <c r="N1" s="17" t="n"/>
+      <c r="O1" s="17" t="n"/>
+      <c r="P1" s="16" t="inlineStr">
+        <is>
+          <t>📞 CONTATTI / SOCIAL</t>
+        </is>
+      </c>
+      <c r="Q1" s="17" t="n"/>
+      <c r="R1" s="17" t="n"/>
+      <c r="S1" s="17" t="n"/>
+      <c r="T1" s="17" t="n"/>
+      <c r="U1" s="17" t="n"/>
+      <c r="V1" s="17" t="n"/>
+      <c r="W1" s="17" t="n"/>
+      <c r="X1" s="16" t="inlineStr">
+        <is>
+          <t>🤝 B2B</t>
+        </is>
+      </c>
+      <c r="Y1" s="17" t="n"/>
+      <c r="Z1" s="17" t="n"/>
+      <c r="AA1" s="16" t="inlineStr">
+        <is>
+          <t>📊 STATO</t>
+        </is>
+      </c>
+      <c r="AB1" s="17" t="n"/>
+      <c r="AC1" s="17" t="n"/>
+      <c r="AD1" s="17" t="n"/>
+      <c r="AE1" s="17" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="E2" s="18" t="inlineStr">
+        <is>
+          <t>borough_id</t>
+        </is>
+      </c>
+      <c r="F2" s="18" t="inlineStr">
+        <is>
+          <t>address_full</t>
+        </is>
+      </c>
+      <c r="G2" s="18" t="inlineStr">
+        <is>
+          <t>coordinates_lat</t>
+        </is>
+      </c>
+      <c r="H2" s="18" t="inlineStr">
+        <is>
+          <t>coordinates_lng</t>
+        </is>
+      </c>
+      <c r="I2" s="18" t="inlineStr">
+        <is>
+          <t>description_short</t>
+        </is>
+      </c>
+      <c r="J2" s="18" t="inlineStr">
+        <is>
+          <t>description_long</t>
+        </is>
+      </c>
+      <c r="K2" s="18" t="inlineStr">
+        <is>
+          <t>tagline</t>
+        </is>
+      </c>
+      <c r="L2" s="18" t="inlineStr">
+        <is>
+          <t>cuisine_type</t>
+        </is>
+      </c>
+      <c r="M2" s="18" t="inlineStr">
+        <is>
+          <t>price_range</t>
+        </is>
+      </c>
+      <c r="N2" s="18" t="inlineStr">
+        <is>
+          <t>seats_indoor</t>
+        </is>
+      </c>
+      <c r="O2" s="18" t="inlineStr">
+        <is>
+          <t>seats_outdoor</t>
+        </is>
+      </c>
+      <c r="P2" s="18" t="inlineStr">
+        <is>
+          <t>opening_hours</t>
+        </is>
+      </c>
+      <c r="Q2" s="18" t="inlineStr">
+        <is>
+          <t>closing_day</t>
+        </is>
+      </c>
+      <c r="R2" s="18" t="inlineStr">
+        <is>
+          <t>specialties</t>
+        </is>
+      </c>
+      <c r="S2" s="18" t="inlineStr">
+        <is>
+          <t>menu_highlights</t>
+        </is>
+      </c>
+      <c r="T2" s="18" t="inlineStr">
+        <is>
+          <t>contact_email</t>
+        </is>
+      </c>
+      <c r="U2" s="18" t="inlineStr">
+        <is>
+          <t>contact_phone</t>
+        </is>
+      </c>
+      <c r="V2" s="18" t="inlineStr">
+        <is>
+          <t>website_url</t>
+        </is>
+      </c>
+      <c r="W2" s="18" t="inlineStr">
+        <is>
+          <t>social_instagram</t>
+        </is>
+      </c>
+      <c r="X2" s="18" t="inlineStr">
+        <is>
+          <t>social_facebook</t>
+        </is>
+      </c>
+      <c r="Y2" s="18" t="inlineStr">
+        <is>
+          <t>booking_url</t>
+        </is>
+      </c>
+      <c r="Z2" s="18" t="inlineStr">
+        <is>
+          <t>accepts_groups</t>
+        </is>
+      </c>
+      <c r="AA2" s="18" t="inlineStr">
+        <is>
+          <t>max_group_size</t>
+        </is>
+      </c>
+      <c r="AB2" s="18" t="inlineStr">
+        <is>
+          <t>b2b_open_for_contact</t>
+        </is>
+      </c>
+      <c r="AC2" s="18" t="inlineStr">
+        <is>
+          <t>b2b_interests</t>
+        </is>
+      </c>
+      <c r="AD2" s="18" t="inlineStr">
+        <is>
+          <t>is_active</t>
+        </is>
+      </c>
+      <c r="AE2" s="18" t="inlineStr">
+        <is>
+          <t>is_featured</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+Es: ristorante-la-taverna-lacedonia</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+URL-friendly. Es: taverna-irpinia-lacedonia</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+Nome del locale</t>
+        </is>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+RISTORANTE / TRATTORIA / PIZZERIA / AGRITURISMO / ENOTECA / BAR / OSTERIA</t>
+        </is>
+      </c>
+      <c r="E3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+ID del borgo. Es: lacedonia</t>
+        </is>
+      </c>
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+Indirizzo completo. Es: Via Roma 1, 83046 Lacedonia (AV)</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+Latitudine GPS. Es: 41.0472</t>
+        </is>
+      </c>
+      <c r="H3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+Longitudine GPS. Es: 15.4297</t>
+        </is>
+      </c>
+      <c r="I3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+Per card (max 160 caratteri)</t>
+        </is>
+      </c>
+      <c r="J3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+Pagina dettaglio (max 800 caratteri)</t>
+        </is>
+      </c>
+      <c r="K3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+Slogan breve (max 80 caratteri)</t>
+        </is>
+      </c>
+      <c r="L3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+Es: Tradizionale Irpina, Pizza, Pesce, Gourmet</t>
+        </is>
+      </c>
+      <c r="M3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+BUDGET / MEDIO / ALTO / GOURMET</t>
+        </is>
+      </c>
+      <c r="N3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+Posti interni</t>
+        </is>
+      </c>
+      <c r="O3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+Posti esterni/terrazza</t>
+        </is>
+      </c>
+      <c r="P3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+Es: Mar-Dom 12:00-15:00, 19:00-23:00</t>
+        </is>
+      </c>
+      <c r="Q3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+Es: Lunedi</t>
+        </is>
+      </c>
+      <c r="R3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+Piatti tipici separati da virgola</t>
+        </is>
+      </c>
+      <c r="S3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+Piatti consigliati separati da |</t>
+        </is>
+      </c>
+      <c r="T3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+Email del locale</t>
+        </is>
+      </c>
+      <c r="U3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+Telefono. Es: +39 0827 12345</t>
+        </is>
+      </c>
+      <c r="V3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+URL sito web</t>
+        </is>
+      </c>
+      <c r="W3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+URL o @handle Instagram</t>
+        </is>
+      </c>
+      <c r="X3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+URL pagina Facebook</t>
+        </is>
+      </c>
+      <c r="Y3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+URL prenotazione (TheFork, Google, proprio sito)</t>
+        </is>
+      </c>
+      <c r="Z3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+SI / NO</t>
+        </is>
+      </c>
+      <c r="AA3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+Max persone per gruppi/eventi</t>
+        </is>
+      </c>
+      <c r="AB3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+SI / NO — disponibile per contatti B2B</t>
+        </is>
+      </c>
+      <c r="AC3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+Es: Forniture locali, Catering, Eventi, Gruppi turistici</t>
+        </is>
+      </c>
+      <c r="AD3" s="19" t="inlineStr">
+        <is>
+          <t>✦ OBBLIGATORIO
+SI / NO</t>
+        </is>
+      </c>
+      <c r="AE3" s="19" t="inlineStr">
+        <is>
+          <t>○ Facoltativo
+SI / NO — metti in evidenza</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>trattoria-del-borgo-lacedonia</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>trattoria-del-borgo-lacedonia</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Trattoria del Borgo</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>TRATTORIA</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>lacedonia</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>Via Roma 23, 83046 Lacedonia (AV)</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="n">
+        <v>41.0472</v>
+      </c>
+      <c r="H4" s="20" t="n">
+        <v>15.4297</v>
+      </c>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>Cucina tradizionale irpina nel cuore del centro storico di Lacedonia, con piatti della nonna e prodotti a km zero.</t>
+        </is>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>La Trattoria del Borgo è il luogo dove la cucina irpina vive nella sua forma più autentica. Situata nel centro storico di Lacedonia, tra le antiche "strette" medievali, propone un menu che cambia con le stagioni: fusilli al ferretto con ragù di castrato, zuppe di legumi con cotiche, caciocavallo podolico alla piastra, e i dolci natalizi della tradizione lacedoniese. Tutti gli ingredienti provengono da produttori locali e dall'orto di famiglia. In estate si mangia nella terrazza panoramica con vista sulla Valle del Calaggio.</t>
+        </is>
+      </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>I sapori autentici dell'Irpinia a tavola</t>
+        </is>
+      </c>
+      <c r="L4" s="20" t="inlineStr">
+        <is>
+          <t>Tradizionale Irpina</t>
+        </is>
+      </c>
+      <c r="M4" s="20" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="N4" s="20" t="n">
+        <v>40</v>
+      </c>
+      <c r="O4" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="P4" s="20" t="inlineStr">
+        <is>
+          <t>Mar-Dom 12:00-15:00, 19:00-22:30</t>
+        </is>
+      </c>
+      <c r="Q4" s="20" t="inlineStr">
+        <is>
+          <t>Lunedi</t>
+        </is>
+      </c>
+      <c r="R4" s="20" t="inlineStr">
+        <is>
+          <t>Fusilli al ferretto con ragù di castrato, Caciocavallo Podolico alla piastra, Zuppa di legumi irpini, Dolci natalizi lacedoniesi</t>
+        </is>
+      </c>
+      <c r="S4" s="20" t="inlineStr">
+        <is>
+          <t>Antipasto del pastore (salumi, formaggi, sottoli)|Fusilli al ragù di castrato|Agnello alla brace con patate|Torta di castagne</t>
+        </is>
+      </c>
+      <c r="T4" s="20" t="inlineStr">
+        <is>
+          <t>info@trattoriadelborgo.it</t>
+        </is>
+      </c>
+      <c r="U4" s="20" t="inlineStr">
+        <is>
+          <t>+39 0827 85100</t>
+        </is>
+      </c>
+      <c r="V4" s="20" t="inlineStr"/>
+      <c r="W4" s="20" t="inlineStr">
+        <is>
+          <t>@trattoriadelborgo</t>
+        </is>
+      </c>
+      <c r="X4" s="20" t="inlineStr"/>
+      <c r="Y4" s="20" t="inlineStr"/>
+      <c r="Z4" s="20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AA4" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC4" s="20" t="inlineStr">
+        <is>
+          <t>Forniture locali, Gruppi turistici, Catering eventi</t>
+        </is>
+      </c>
+      <c r="AD4" s="20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AE4" s="20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:S53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -12787,25 +12560,107 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
-      <c r="P4" s="5" t="n"/>
-      <c r="Q4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
-      <c r="S4" s="5" t="n"/>
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>lacedonia</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Lacedonia</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Terra di Storia, Terra di Miracoli, Terra di Cultura</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Borgo autentico dell'Alta Irpinia dove 13.000 anni di storia vivono tra vicoli medievali, palazzi nobiliari e tradizioni millenarie. Arroccato a 732 m, Lacedonia custodisce un patrimonio unico tra archeologia, fede e innovazione digitale.</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>Lacedonia: Borgo Autentico tra Storia Millenaria e Innovazione Digitale
+Lacedonia si svela al visitatore come un borgo autentico dell'Alta Irpinia dove 13.000 anni di storia continuano a vivere tra vicoli medievali, palazzi nobiliari e tradizioni che il tempo non ha spezzato. Arroccato a 732 metri di altitudine, questo straordinario comune custodisce un'identità profonda che affonda le radici nell'antichità più remota e si proietta con determinazione verso il futuro.
+Terra di Storia: dall'Antica Aquilonia ai Romani
+Il patrimonio archeologico di Lacedonia affonda le radici nella civiltà sannitica, quando il territorio era parte dell'importante municipium romano di Aquilonia, centro strategico nell'organizzazione amministrativa e militare dell'Italia meridionale. I reperti romani rinvenuti nel corso dei secoli testimoniano la ricchezza e l'importanza di questo antico insediamento, che controllava i collegamenti tra la Campania interna e la Puglia. Le oltre 150 grotte tufacee abitate sin da 13.000 anni fa raccontano una continuità insediativa eccezionale, mentre il centro storico con le sue caratteristiche "strette" medievali che si intrecciano come un labirinto di pietra conserva l'atmosfera di un borgo dove il tempo rallenta, permettendo di riscoprire ritmi più umani e connessioni profonde.
+Terra di Miracoli: San Gerardo Maiella e il Pozzo Prodigioso
+Lacedonia è universalmente riconosciuta come Terra di Miracoli, legata indissolubilmente alla figura di San Gerardo Maiella, santo patrono delle mamme e dei bambini, venerato in tutto il mondo cattolico. Il celebre Pozzo del Miracolo rappresenta uno dei luoghi di pellegrinaggio più significativi dell'Irpinia, dove la tradizione popolare tramanda eventi prodigiosi legati al passaggio del santo. Il Palazzo Vescovile, che ospitò San Gerardo durante i suoi soggiorni a Lacedonia, è diventato meta di devozione per migliaia di fedeli che ogni anno giungono da ogni parte d'Italia e del mondo per rendere omaggio al santo e attingere alla spiritualità profonda che permea questi luoghi.
+Terra di Cultura: Francesco De Sanctis e l'Illuminismo Meridionale
+Lacedonia si distingue come Terra di Cultura grazie alla presenza dell'Istituto Magistrale fondato da Francesco De Sanctis nel 1878, uno dei primi esempi di scuola nell'Italia post-unificazione e simbolo dell'impegno per l'emancipazione culturale del Mezzogiorno. De Sanctis, eminente critico letterario, filosofo e uomo politico italiano, scelse la sua terra d'origine per realizzare un progetto educativo rivoluzionario: formare nuovi maestri elementari per diffondere il sapere nelle zone più periferiche del Sud Italia.
+Patrimonio Religioso e Artistico di Eccellenza
+La Concattedrale di Santa Maria Assunta domina il panorama con la sua imponente architettura barocca del XVII secolo. Il Museo Diocesano conserva preziose testimonianze d'arte sacra. La Chiesa di Santa Maria della Cancellata, edificata su un antico tempio romano dedicato alla dea Iside, testimonia la continuità millenaria delle presenze religiose. La leggenda popolare ha donato al territorio un'aura di mistero attraverso la celebre Casa del Diavolo, enigmatica struttura arroccata su una rupe tufacea.
+Eccellenze Culturali Internazionali
+Tra le attrazioni di eccellenza brilla il MAVI (Museo Antropologico Visivo Irpino), istituzione culturale unica a livello internazionale che custodisce 1.801 fotografie scattate nel 1957 dall'antropologo americano Frank Cancian. Questo straordinario archivio visivo documenta la vita quotidiana della comunità contadina irpina degli anni Cinquanta, offrendo un viaggio emozionante in un mondo rurale che rivive nella memoria collettiva.
+Patrimonio Naturalistico e Tradizioni Millenarie
+I Boschi dell'Origlio, con le loro sorgenti minerali dalle proprietà benefiche, sono un polmone verde di straordinaria ricchezza. Due alberi monumentali riconosciuti dalla Regione Campania, il Cerro del Tesoro e il Cerro del Drago, vegliano sul territorio. La Valle del Calaggio, teatro delle antiche guerre sannitiche, offre scenari di rara suggestione. La transumanza, riconosciuta Patrimonio UNESCO nel 2019, rappresenta un elemento identitario di eccezionale valore.
+Eccellenze Enogastronomiche
+Il territorio è rinomato per gli asparagi selvatici di Contrada Forna, lo zafferano irpino, la produzione casearia tradizionale con formaggi di straordinaria qualità e i dolci natalizi tramandati di generazione in generazione. Il territorio si inserisce nel circuito delle grandi produzioni DOCG dell'Irpinia.
+Innovazione Digitale per il Futuro
+Lacedonia si distingue oggi come borgo all'avanguardia nella trasformazione digitale dei territori rurali. Grazie alla piattaforma innovativa sviluppata da InnTour, oltre 150.000 mq del centro storico sono stati mappati con tecnologie di ultima generazione. Scansioni 3D, fotografie panoramiche a 360°, contenuti multimediali immersivi e avatar AI conversazionali permettono di esplorare ogni angolo in un'esperienza che fonde passato e futuro.
+Scopri i sapori, vivi le tradizioni, respira la storia. Benvenuto a Lacedonia, dove ogni pietra racconta e ogni esperienza emoziona.</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>MAVI — Museo Antropologico Visivo Irpino (1.801 foto di Frank Cancian, 1957)</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Terra di Miracoli — San Gerardo Maiella e il Pozzo Prodigioso</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Innovazione Digitale — 150.000 mq mappati in 3D da InnTour</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>MAVI, Museo Diocesano, Concattedrale S. Maria Assunta, Pozzo del Miracolo, Casa del Diavolo, Grotte Tufacee, Boschi dell'Origlio, Valle del Calaggio, Cammino dei Tratturi, Tour Caseificio Podolico</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="n">
+        <v>732</v>
+      </c>
+      <c r="K4" s="15" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="L4" s="15" t="n">
+        <v>2300</v>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>Avellino</t>
+        </is>
+      </c>
+      <c r="N4" s="15" t="inlineStr">
+        <is>
+          <t>Campania</t>
+        </is>
+      </c>
+      <c r="O4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" s="15" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/embed/XhB4SonU7Pw?autoplay=1&amp;mute=1&amp;loop=1&amp;playlist=XhB4SonU7Pw</t>
+        </is>
+      </c>
+      <c r="S4" s="15" t="inlineStr">
+        <is>
+          <t>https://my.treedis.com/tour/lacedonia-vrcerogn</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="n"/>
@@ -13848,7 +13703,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>